<commit_message>
base demand redux with 80 percent scenario
</commit_message>
<xml_diff>
--- a/DATA/demand/antigen_CI_Random_generator.xlsx
+++ b/DATA/demand/antigen_CI_Random_generator.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="590" documentId="11_4A5645C871AEA98286DE389EAFF8EF0F542BC54D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2937F37B-86E6-431C-A5C2-8E05EA8207B0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Diphtheria" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <sheet name="HPV" sheetId="12" r:id="rId12"/>
     <sheet name="Scenario_data" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -336,34 +336,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>313102875.44879305</c:v>
+                  <c:v>346398627.64330411</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>258583571.46928811</c:v>
+                  <c:v>609788409.3365891</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>624735975.81811237</c:v>
+                  <c:v>525550757.40149248</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>698948600.61900103</c:v>
+                  <c:v>518535636.92032444</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>598971578.13990557</c:v>
+                  <c:v>678867528.27629232</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>669938727.58467209</c:v>
+                  <c:v>613151699.66175199</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>858041721.83717883</c:v>
+                  <c:v>745938422.0467608</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>982324516.90472341</c:v>
+                  <c:v>981655245.73239946</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>847096484.22264278</c:v>
+                  <c:v>758121639.38688612</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>699194982.27341413</c:v>
+                  <c:v>1054136692.0376759</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -408,34 +408,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>29353628.074818686</c:v>
+                  <c:v>20840110.913639396</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>32537650.044107866</c:v>
+                  <c:v>33003198.189924993</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>39366857.745121069</c:v>
+                  <c:v>37564948.897706904</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>34343404.950566143</c:v>
+                  <c:v>38297819.090270177</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46741141.994529955</c:v>
+                  <c:v>43196820.504247271</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>31092524.433205169</c:v>
+                  <c:v>40800099.727116153</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>59019489.163654804</c:v>
+                  <c:v>55512117.873587593</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>54156045.118848495</c:v>
+                  <c:v>42130742.493162677</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>48931800.745717496</c:v>
+                  <c:v>51577977.658602305</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>70878049.684350103</c:v>
+                  <c:v>62584548.099562094</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -480,34 +480,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>408745810.96556836</c:v>
+                  <c:v>272373463.40747488</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>424609749.97643918</c:v>
+                  <c:v>483516328.73493004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>421344487.24847007</c:v>
+                  <c:v>289119898.10361594</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>486789456.52070808</c:v>
+                  <c:v>414059893.41429448</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>533594749.31181866</c:v>
+                  <c:v>432718696.23840481</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>516430997.50526792</c:v>
+                  <c:v>648180888.19893277</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>854302314.37320733</c:v>
+                  <c:v>734672167.46613932</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>727522986.83084035</c:v>
+                  <c:v>821487018.30194342</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>813449257.77919173</c:v>
+                  <c:v>817668241.94867456</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>799136936.70137048</c:v>
+                  <c:v>695484711.98491108</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -552,34 +552,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>625302065.02012849</c:v>
+                  <c:v>652096368.2216897</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>706692052.3953979</c:v>
+                  <c:v>674341526.85532749</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>750543450.11648631</c:v>
+                  <c:v>717706771.55113971</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>816565360.60382926</c:v>
+                  <c:v>934898423.3402555</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>970683647.47504902</c:v>
+                  <c:v>910992813.42327571</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1208008489.5923297</c:v>
+                  <c:v>1182799454.738198</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1352307677.5593073</c:v>
+                  <c:v>1384125950.1142042</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1617517085.2339122</c:v>
+                  <c:v>1604956477.0636852</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1625663109.9002686</c:v>
+                  <c:v>1648666503.6256371</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1902813642.1379783</c:v>
+                  <c:v>2003485736.807965</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -624,34 +624,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>650970822.56898654</c:v>
+                  <c:v>580321768.84763432</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>619268075.03400934</c:v>
+                  <c:v>618409157.36515844</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>631788067.9471004</c:v>
+                  <c:v>646864171.13713646</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>691384012.4254334</c:v>
+                  <c:v>675476437.66133559</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>675440352.04472125</c:v>
+                  <c:v>707358024.11453915</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>701056726.73188722</c:v>
+                  <c:v>705923805.05312788</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>676359138.52133548</c:v>
+                  <c:v>677684598.1991353</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>704159366.74474478</c:v>
+                  <c:v>756577838.53838158</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>706345126.76525784</c:v>
+                  <c:v>712522135.88390744</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>722315359.08481681</c:v>
+                  <c:v>744577945.9480027</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -696,34 +696,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>369019997.25248706</c:v>
+                  <c:v>377099079.522255</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>327075398.68409991</c:v>
+                  <c:v>349743008.42086285</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>329416556.92000383</c:v>
+                  <c:v>358828924.65739149</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>360936826.88394058</c:v>
+                  <c:v>384166685.06519914</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>379958217.69572496</c:v>
+                  <c:v>321018131.2935856</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>322281409.03089046</c:v>
+                  <c:v>371783799.60341054</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>402541327.16018939</c:v>
+                  <c:v>361224164.75770944</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>359028892.43529868</c:v>
+                  <c:v>379838866.49923599</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>325242719.89408427</c:v>
+                  <c:v>397507726.06506461</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>421465050.10378128</c:v>
+                  <c:v>400664505.44185388</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -770,34 +770,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>355778692.35009098</c:v>
+                  <c:v>390859091.0957067</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>438002523.10604686</c:v>
+                  <c:v>385955632.35852683</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>389734412.31942236</c:v>
+                  <c:v>323629206.30780774</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>403817107.07063323</c:v>
+                  <c:v>424663649.35197407</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>391327351.94039482</c:v>
+                  <c:v>373482318.40589166</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>452020208.05661857</c:v>
+                  <c:v>358036029.12115455</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>361744045.68037063</c:v>
+                  <c:v>480866833.4064604</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>373964982.33362991</c:v>
+                  <c:v>476777441.9324975</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>427884781.59073621</c:v>
+                  <c:v>438033992.66444403</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>436086533.40796435</c:v>
+                  <c:v>424575883.86303997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -844,34 +844,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>289359717.07491219</c:v>
+                  <c:v>300732688.74825186</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>313363487.12721384</c:v>
+                  <c:v>301138426.85186619</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>343475515.11765915</c:v>
+                  <c:v>352704690.37444395</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>334837340.45689988</c:v>
+                  <c:v>346461019.72448152</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>363884818.47186959</c:v>
+                  <c:v>357200804.05163914</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>357188006.89770454</c:v>
+                  <c:v>312268189.61223459</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>348934285.05260718</c:v>
+                  <c:v>360212222.90886766</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>381549183.42356211</c:v>
+                  <c:v>375709755.60838896</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>409555583.44038814</c:v>
+                  <c:v>397730594.11381888</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>403900578.3239277</c:v>
+                  <c:v>425669766.29332536</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -918,34 +918,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>581839336.02645445</c:v>
+                  <c:v>587059615.91624844</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>649172550.55085421</c:v>
+                  <c:v>711589396.21656442</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>567159776.66132641</c:v>
+                  <c:v>695287580.72666001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>692694739.33496797</c:v>
+                  <c:v>768463061.4913609</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>717832136.94679999</c:v>
+                  <c:v>718238764.86178637</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>834927990.10967553</c:v>
+                  <c:v>753604437.83078837</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>803843472.5752368</c:v>
+                  <c:v>839210342.65936148</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>797130260.47852981</c:v>
+                  <c:v>804551762.56089425</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>830331997.11825132</c:v>
+                  <c:v>881493869.87954855</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>954723224.3480581</c:v>
+                  <c:v>859201436.88993907</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -992,34 +992,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>28813061.981344361</c:v>
+                  <c:v>27250263.793651372</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>34513806.317383148</c:v>
+                  <c:v>33604048.931154117</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40246926.621811047</c:v>
+                  <c:v>42521002.697570607</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45395490.20459792</c:v>
+                  <c:v>46309572.189586237</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>56830506.861267693</c:v>
+                  <c:v>55327907.464503817</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>59228362.113960996</c:v>
+                  <c:v>59490904.512177654</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67963050.336423963</c:v>
+                  <c:v>65506111.644410707</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>73398426.17083995</c:v>
+                  <c:v>71881059.651827395</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>83823211.643525869</c:v>
+                  <c:v>79714888.524668857</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>89659414.119553238</c:v>
+                  <c:v>87510069.202634826</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1066,34 +1066,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>212356179.18269354</c:v>
+                  <c:v>203184261.34051713</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>228002743.31291083</c:v>
+                  <c:v>193888232.76516005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>226863050.68823063</c:v>
+                  <c:v>237913229.93208605</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>299343945.00113678</c:v>
+                  <c:v>244389697.47415298</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>316684901.98480678</c:v>
+                  <c:v>349629111.22157079</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>372084322.09227526</c:v>
+                  <c:v>427250110.0740537</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>447559080.14459324</c:v>
+                  <c:v>457142117.25461364</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>524263673.48202568</c:v>
+                  <c:v>507144865.37986726</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>600000823.35737109</c:v>
+                  <c:v>647901558.97098541</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>743326072.76503897</c:v>
+                  <c:v>737219212.85431552</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1140,34 +1140,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>234292637.76584065</c:v>
+                  <c:v>211403260.01881739</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>251340614.35331798</c:v>
+                  <c:v>251439115.74413413</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>286798993.08894235</c:v>
+                  <c:v>270272253.56533325</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>318702438.85792321</c:v>
+                  <c:v>317723220.10685098</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>337336416.02681231</c:v>
+                  <c:v>337170221.39178747</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>368705685.98718059</c:v>
+                  <c:v>365214546.95532507</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>408722386.12393236</c:v>
+                  <c:v>395976114.41627443</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>451798991.30340707</c:v>
+                  <c:v>449048557.10372937</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>478974333.83229929</c:v>
+                  <c:v>495827019.50174165</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>425893971.36649722</c:v>
+                  <c:v>418569031.30105716</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3080,43 +3080,43 @@
       </c>
       <c r="B2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C2,Measles!$D$2)</f>
-        <v>313102875.44879305</v>
+        <v>346398627.64330411</v>
       </c>
       <c r="C2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C3,Measles!$D$2)</f>
-        <v>258583571.46928811</v>
+        <v>609788409.3365891</v>
       </c>
       <c r="D2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C4,Measles!$D$2)</f>
-        <v>624735975.81811237</v>
+        <v>525550757.40149248</v>
       </c>
       <c r="E2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C5,Measles!$D$2)</f>
-        <v>698948600.61900103</v>
+        <v>518535636.92032444</v>
       </c>
       <c r="F2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C6,Measles!$D$2)</f>
-        <v>598971578.13990557</v>
+        <v>678867528.27629232</v>
       </c>
       <c r="G2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C7,Measles!$D$2)</f>
-        <v>669938727.58467209</v>
+        <v>613151699.66175199</v>
       </c>
       <c r="H2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C8,Measles!$D$2)</f>
-        <v>858041721.83717883</v>
+        <v>745938422.0467608</v>
       </c>
       <c r="I2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C9,Measles!$D$2)</f>
-        <v>982324516.90472341</v>
+        <v>981655245.73239946</v>
       </c>
       <c r="J2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C10,Measles!$D$2)</f>
-        <v>847096484.22264278</v>
+        <v>758121639.38688612</v>
       </c>
       <c r="K2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C11,Measles!$D$2)</f>
-        <v>699194982.27341413</v>
+        <v>1054136692.0376759</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
@@ -3125,43 +3125,43 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C2,Mumps!$D$2)</f>
-        <v>29353628.074818686</v>
+        <v>20840110.913639396</v>
       </c>
       <c r="C3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C3,Mumps!$D$2)</f>
-        <v>32537650.044107866</v>
+        <v>33003198.189924993</v>
       </c>
       <c r="D3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C4,Mumps!$D$2)</f>
-        <v>39366857.745121069</v>
+        <v>37564948.897706904</v>
       </c>
       <c r="E3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C5,Mumps!$D$2)</f>
-        <v>34343404.950566143</v>
+        <v>38297819.090270177</v>
       </c>
       <c r="F3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C6,Mumps!$D$2)</f>
-        <v>46741141.994529955</v>
+        <v>43196820.504247271</v>
       </c>
       <c r="G3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C7,Mumps!$D$2)</f>
-        <v>31092524.433205169</v>
+        <v>40800099.727116153</v>
       </c>
       <c r="H3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C8,Mumps!$D$2)</f>
-        <v>59019489.163654804</v>
+        <v>55512117.873587593</v>
       </c>
       <c r="I3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C9,Mumps!$D$2)</f>
-        <v>54156045.118848495</v>
+        <v>42130742.493162677</v>
       </c>
       <c r="J3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C10,Mumps!$D$2)</f>
-        <v>48931800.745717496</v>
+        <v>51577977.658602305</v>
       </c>
       <c r="K3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C11,Mumps!$D$2)</f>
-        <v>70878049.684350103</v>
+        <v>62584548.099562094</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -3170,43 +3170,43 @@
       </c>
       <c r="B4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C2,Rubella!$D$2)</f>
-        <v>408745810.96556836</v>
+        <v>272373463.40747488</v>
       </c>
       <c r="C4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C3,Rubella!$D$2)</f>
-        <v>424609749.97643918</v>
+        <v>483516328.73493004</v>
       </c>
       <c r="D4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C4,Rubella!$D$2)</f>
-        <v>421344487.24847007</v>
+        <v>289119898.10361594</v>
       </c>
       <c r="E4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C5,Rubella!$D$2)</f>
-        <v>486789456.52070808</v>
+        <v>414059893.41429448</v>
       </c>
       <c r="F4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C6,Rubella!$D$2)</f>
-        <v>533594749.31181866</v>
+        <v>432718696.23840481</v>
       </c>
       <c r="G4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C7,Rubella!$D$2)</f>
-        <v>516430997.50526792</v>
+        <v>648180888.19893277</v>
       </c>
       <c r="H4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C8,Rubella!$D$2)</f>
-        <v>854302314.37320733</v>
+        <v>734672167.46613932</v>
       </c>
       <c r="I4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C9,Rubella!$D$2)</f>
-        <v>727522986.83084035</v>
+        <v>821487018.30194342</v>
       </c>
       <c r="J4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C10,Rubella!$D$2)</f>
-        <v>813449257.77919173</v>
+        <v>817668241.94867456</v>
       </c>
       <c r="K4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C11,Rubella!$D$2)</f>
-        <v>799136936.70137048</v>
+        <v>695484711.98491108</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -3215,43 +3215,43 @@
       </c>
       <c r="B5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C2,Diphtheria!$D$2)</f>
-        <v>625302065.02012849</v>
+        <v>652096368.2216897</v>
       </c>
       <c r="C5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C3,Diphtheria!$D$2)</f>
-        <v>706692052.3953979</v>
+        <v>674341526.85532749</v>
       </c>
       <c r="D5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C4,Diphtheria!$D$2)</f>
-        <v>750543450.11648631</v>
+        <v>717706771.55113971</v>
       </c>
       <c r="E5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C5,Diphtheria!$D$2)</f>
-        <v>816565360.60382926</v>
+        <v>934898423.3402555</v>
       </c>
       <c r="F5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C6,Diphtheria!$D$2)</f>
-        <v>970683647.47504902</v>
+        <v>910992813.42327571</v>
       </c>
       <c r="G5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C8,Diphtheria!$D$2)</f>
-        <v>1208008489.5923297</v>
+        <v>1182799454.738198</v>
       </c>
       <c r="H5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C9,Diphtheria!$D$2)</f>
-        <v>1352307677.5593073</v>
+        <v>1384125950.1142042</v>
       </c>
       <c r="I5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1617517085.2339122</v>
+        <v>1604956477.0636852</v>
       </c>
       <c r="J5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1625663109.9002686</v>
+        <v>1648666503.6256371</v>
       </c>
       <c r="K5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C11,Diphtheria!$D$2)</f>
-        <v>1902813642.1379783</v>
+        <v>2003485736.807965</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
@@ -3260,43 +3260,43 @@
       </c>
       <c r="B6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C2,Tetanus!$D$2)</f>
-        <v>650970822.56898654</v>
+        <v>580321768.84763432</v>
       </c>
       <c r="C6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C3,Tetanus!$D$2)</f>
-        <v>619268075.03400934</v>
+        <v>618409157.36515844</v>
       </c>
       <c r="D6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C4,Tetanus!$D$2)</f>
-        <v>631788067.9471004</v>
+        <v>646864171.13713646</v>
       </c>
       <c r="E6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C5,Tetanus!$D$2)</f>
-        <v>691384012.4254334</v>
+        <v>675476437.66133559</v>
       </c>
       <c r="F6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C6,Tetanus!$D$2)</f>
-        <v>675440352.04472125</v>
+        <v>707358024.11453915</v>
       </c>
       <c r="G6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C7,Tetanus!$D$2)</f>
-        <v>701056726.73188722</v>
+        <v>705923805.05312788</v>
       </c>
       <c r="H6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C8,Tetanus!$D$2)</f>
-        <v>676359138.52133548</v>
+        <v>677684598.1991353</v>
       </c>
       <c r="I6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C9,Tetanus!$D$2)</f>
-        <v>704159366.74474478</v>
+        <v>756577838.53838158</v>
       </c>
       <c r="J6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C10,Tetanus!$D$2)</f>
-        <v>706345126.76525784</v>
+        <v>712522135.88390744</v>
       </c>
       <c r="K6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C11,Tetanus!$D$2)</f>
-        <v>722315359.08481681</v>
+        <v>744577945.9480027</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -3305,43 +3305,43 @@
       </c>
       <c r="B7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>369019997.25248706</v>
+        <v>377099079.522255</v>
       </c>
       <c r="C7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>327075398.68409991</v>
+        <v>349743008.42086285</v>
       </c>
       <c r="D7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C4,Pertussis!$D$2)</f>
-        <v>329416556.92000383</v>
+        <v>358828924.65739149</v>
       </c>
       <c r="E7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C5,Pertussis!$D$2)</f>
-        <v>360936826.88394058</v>
+        <v>384166685.06519914</v>
       </c>
       <c r="F7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C6,Pertussis!$D$2)</f>
-        <v>379958217.69572496</v>
+        <v>321018131.2935856</v>
       </c>
       <c r="G7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C7,Pertussis!$D$2)</f>
-        <v>322281409.03089046</v>
+        <v>371783799.60341054</v>
       </c>
       <c r="H7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C8,Pertussis!$D$2)</f>
-        <v>402541327.16018939</v>
+        <v>361224164.75770944</v>
       </c>
       <c r="I7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C9,Pertussis!$D$2)</f>
-        <v>359028892.43529868</v>
+        <v>379838866.49923599</v>
       </c>
       <c r="J7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C10,Pertussis!$D$2)</f>
-        <v>325242719.89408427</v>
+        <v>397507726.06506461</v>
       </c>
       <c r="K7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C11,Pertussis!$D$2)</f>
-        <v>421465050.10378128</v>
+        <v>400664505.44185388</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
@@ -3350,43 +3350,43 @@
       </c>
       <c r="B8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C2,Hepatitis_B!$D$2)</f>
-        <v>355778692.35009098</v>
+        <v>390859091.0957067</v>
       </c>
       <c r="C8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C3,Hepatitis_B!$D$2)</f>
-        <v>438002523.10604686</v>
+        <v>385955632.35852683</v>
       </c>
       <c r="D8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C4,Hepatitis_B!$D$2)</f>
-        <v>389734412.31942236</v>
+        <v>323629206.30780774</v>
       </c>
       <c r="E8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C5,Hepatitis_B!$D$2)</f>
-        <v>403817107.07063323</v>
+        <v>424663649.35197407</v>
       </c>
       <c r="F8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C6,Hepatitis_B!$D$2)</f>
-        <v>391327351.94039482</v>
+        <v>373482318.40589166</v>
       </c>
       <c r="G8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C7,Hepatitis_B!$D$2)</f>
-        <v>452020208.05661857</v>
+        <v>358036029.12115455</v>
       </c>
       <c r="H8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C8,Hepatitis_B!$D$2)</f>
-        <v>361744045.68037063</v>
+        <v>480866833.4064604</v>
       </c>
       <c r="I8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C9,Hepatitis_B!$D$2)</f>
-        <v>373964982.33362991</v>
+        <v>476777441.9324975</v>
       </c>
       <c r="J8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C10,Hepatitis_B!$D$2)</f>
-        <v>427884781.59073621</v>
+        <v>438033992.66444403</v>
       </c>
       <c r="K8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,Hepatitis_B!$D$2)</f>
-        <v>436086533.40796435</v>
+        <v>424575883.86303997</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
@@ -3395,43 +3395,43 @@
       </c>
       <c r="B9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C2,Hib!$D$2)</f>
-        <v>289359717.07491219</v>
+        <v>300732688.74825186</v>
       </c>
       <c r="C9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C3,Hib!$D$2)</f>
-        <v>313363487.12721384</v>
+        <v>301138426.85186619</v>
       </c>
       <c r="D9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C4,Hib!$D$2)</f>
-        <v>343475515.11765915</v>
+        <v>352704690.37444395</v>
       </c>
       <c r="E9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C5,Hib!$D$2)</f>
-        <v>334837340.45689988</v>
+        <v>346461019.72448152</v>
       </c>
       <c r="F9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C6,Hib!$D$2)</f>
-        <v>363884818.47186959</v>
+        <v>357200804.05163914</v>
       </c>
       <c r="G9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C7,Hib!$D$2)</f>
-        <v>357188006.89770454</v>
+        <v>312268189.61223459</v>
       </c>
       <c r="H9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C8,Hib!$D$2)</f>
-        <v>348934285.05260718</v>
+        <v>360212222.90886766</v>
       </c>
       <c r="I9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C9,Hib!$D$2)</f>
-        <v>381549183.42356211</v>
+        <v>375709755.60838896</v>
       </c>
       <c r="J9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C10,Hib!$D$2)</f>
-        <v>409555583.44038814</v>
+        <v>397730594.11381888</v>
       </c>
       <c r="K9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C11,Hib!$D$2)</f>
-        <v>403900578.3239277</v>
+        <v>425669766.29332536</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
@@ -3440,43 +3440,43 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C2,Polio!$D$2)</f>
-        <v>581839336.02645445</v>
+        <v>587059615.91624844</v>
       </c>
       <c r="C10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C3,Polio!$D$2)</f>
-        <v>649172550.55085421</v>
+        <v>711589396.21656442</v>
       </c>
       <c r="D10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C4,Polio!$D$2)</f>
-        <v>567159776.66132641</v>
+        <v>695287580.72666001</v>
       </c>
       <c r="E10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C5,Polio!$D$2)</f>
-        <v>692694739.33496797</v>
+        <v>768463061.4913609</v>
       </c>
       <c r="F10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C6,Polio!$D$2)</f>
-        <v>717832136.94679999</v>
+        <v>718238764.86178637</v>
       </c>
       <c r="G10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C7,Polio!$D$2)</f>
-        <v>834927990.10967553</v>
+        <v>753604437.83078837</v>
       </c>
       <c r="H10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C8,Polio!$D$2)</f>
-        <v>803843472.5752368</v>
+        <v>839210342.65936148</v>
       </c>
       <c r="I10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C9,Polio!$D$2)</f>
-        <v>797130260.47852981</v>
+        <v>804551762.56089425</v>
       </c>
       <c r="J10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C10,Polio!$D$2)</f>
-        <v>830331997.11825132</v>
+        <v>881493869.87954855</v>
       </c>
       <c r="K10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C11,Polio!$D$2)</f>
-        <v>954723224.3480581</v>
+        <v>859201436.88993907</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
@@ -3485,43 +3485,43 @@
       </c>
       <c r="B11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C2,HPV!$D$2)</f>
-        <v>28813061.981344361</v>
+        <v>27250263.793651372</v>
       </c>
       <c r="C11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C3,HPV!$D$2)</f>
-        <v>34513806.317383148</v>
+        <v>33604048.931154117</v>
       </c>
       <c r="D11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C4,HPV!$D$2)</f>
-        <v>40246926.621811047</v>
+        <v>42521002.697570607</v>
       </c>
       <c r="E11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C5,HPV!$D$2)</f>
-        <v>45395490.20459792</v>
+        <v>46309572.189586237</v>
       </c>
       <c r="F11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C6,HPV!$D$2)</f>
-        <v>56830506.861267693</v>
+        <v>55327907.464503817</v>
       </c>
       <c r="G11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C7,HPV!$D$2)</f>
-        <v>59228362.113960996</v>
+        <v>59490904.512177654</v>
       </c>
       <c r="H11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C8,HPV!$D$2)</f>
-        <v>67963050.336423963</v>
+        <v>65506111.644410707</v>
       </c>
       <c r="I11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C9,HPV!$D$2)</f>
-        <v>73398426.17083995</v>
+        <v>71881059.651827395</v>
       </c>
       <c r="J11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C10,HPV!$D$2)</f>
-        <v>83823211.643525869</v>
+        <v>79714888.524668857</v>
       </c>
       <c r="K11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C11,HPV!$D$2)</f>
-        <v>89659414.119553238</v>
+        <v>87510069.202634826</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
@@ -3530,43 +3530,43 @@
       </c>
       <c r="B12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C2,Rotavirus!$D$2)</f>
-        <v>212356179.18269354</v>
+        <v>203184261.34051713</v>
       </c>
       <c r="C12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C3,Rotavirus!$D$2)</f>
-        <v>228002743.31291083</v>
+        <v>193888232.76516005</v>
       </c>
       <c r="D12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C4,Rotavirus!$D$2)</f>
-        <v>226863050.68823063</v>
+        <v>237913229.93208605</v>
       </c>
       <c r="E12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C5,Rotavirus!$D$2)</f>
-        <v>299343945.00113678</v>
+        <v>244389697.47415298</v>
       </c>
       <c r="F12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C6,Rotavirus!$D$2)</f>
-        <v>316684901.98480678</v>
+        <v>349629111.22157079</v>
       </c>
       <c r="G12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C7,Rotavirus!$D$2)</f>
-        <v>372084322.09227526</v>
+        <v>427250110.0740537</v>
       </c>
       <c r="H12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C8,Rotavirus!$D$2)</f>
-        <v>447559080.14459324</v>
+        <v>457142117.25461364</v>
       </c>
       <c r="I12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C9,Rotavirus!$D$2)</f>
-        <v>524263673.48202568</v>
+        <v>507144865.37986726</v>
       </c>
       <c r="J12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C10,Rotavirus!$D$2)</f>
-        <v>600000823.35737109</v>
+        <v>647901558.97098541</v>
       </c>
       <c r="K12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C11,Rotavirus!$D$2)</f>
-        <v>743326072.76503897</v>
+        <v>737219212.85431552</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
@@ -3575,43 +3575,43 @@
       </c>
       <c r="B13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C2,PCV!$D$2)</f>
-        <v>234292637.76584065</v>
+        <v>209977032.97029382</v>
       </c>
       <c r="C13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C3,PCV!$D$2)</f>
-        <v>251340614.35331798</v>
+        <v>251439115.74413413</v>
       </c>
       <c r="D13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C4,PCV!$D$2)</f>
-        <v>286798993.08894235</v>
+        <v>270272253.56533325</v>
       </c>
       <c r="E13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C5,PCV!$D$2)</f>
-        <v>318702438.85792321</v>
+        <v>317723220.10685098</v>
       </c>
       <c r="F13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C6,PCV!$D$2)</f>
-        <v>337336416.02681231</v>
+        <v>337170221.39178747</v>
       </c>
       <c r="G13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C7,PCV!$D$2)</f>
-        <v>368705685.98718059</v>
+        <v>365214546.95532507</v>
       </c>
       <c r="H13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C8,PCV!$D$2)</f>
-        <v>408722386.12393236</v>
+        <v>395976114.41627443</v>
       </c>
       <c r="I13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C9,PCV!$D$2)</f>
-        <v>451798991.30340707</v>
+        <v>449048557.10372937</v>
       </c>
       <c r="J13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C10,PCV!$D$2)</f>
-        <v>478974333.83229929</v>
+        <v>495827019.50174165</v>
       </c>
       <c r="K13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,PCV!$D$2)</f>
-        <v>425893971.36649722</v>
+        <v>418569031.30105716</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
@@ -3620,43 +3620,43 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(B2&gt;Measles!B2,Measles!B2,IF(Scenario_data!B2 &lt;Measles!A2,Measles!A2,Scenario_data!B2))</f>
-        <v>313102875.44879305</v>
+        <v>346398627.64330411</v>
       </c>
       <c r="C15" s="7">
         <f ca="1">IF(C2&gt;Measles!B3,Measles!B3,IF(Scenario_data!C2 &lt;Measles!A3,Measles!A3,Scenario_data!C2))</f>
-        <v>258583571.46928811</v>
+        <v>609788409.3365891</v>
       </c>
       <c r="D15" s="7">
         <f ca="1">IF(D2&gt;Measles!B4,Measles!B4,IF(Scenario_data!D2 &lt;Measles!A4,Measles!A4,Scenario_data!D2))</f>
-        <v>624735975.81811237</v>
+        <v>525550757.40149248</v>
       </c>
       <c r="E15" s="7">
         <f ca="1">IF(E2&gt;Measles!B5,Measles!B5,IF(Scenario_data!E2 &lt;Measles!A5,Measles!A5,Scenario_data!E2))</f>
-        <v>698948600.61900103</v>
+        <v>518535636.92032444</v>
       </c>
       <c r="F15" s="7">
         <f ca="1">IF(F2&gt;Measles!B6,Measles!B6,IF(Scenario_data!F2 &lt;Measles!A6,Measles!A6,Scenario_data!F2))</f>
-        <v>598971578.13990557</v>
+        <v>678867528.27629232</v>
       </c>
       <c r="G15" s="7">
         <f ca="1">IF(G2&gt;Measles!B7,Measles!B7,IF(Scenario_data!G2 &lt;Measles!A7,Measles!A7,Scenario_data!G2))</f>
-        <v>669938727.58467209</v>
+        <v>613151699.66175199</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">IF(H2&gt;Measles!B8,Measles!B8,IF(Scenario_data!H2 &lt;Measles!A8,Measles!A8,Scenario_data!H2))</f>
-        <v>858041721.83717883</v>
+        <v>745938422.0467608</v>
       </c>
       <c r="I15" s="7">
         <f ca="1">IF(I2&gt;Measles!B9,Measles!B9,IF(Scenario_data!I2 &lt;Measles!A9,Measles!A9,Scenario_data!I2))</f>
-        <v>982324516.90472341</v>
+        <v>981655245.73239946</v>
       </c>
       <c r="J15" s="7">
         <f ca="1">IF(J2&gt;Measles!B10,Measles!B10,IF(Scenario_data!J2 &lt;Measles!A10,Measles!A10,Scenario_data!J2))</f>
-        <v>847096484.22264278</v>
+        <v>758121639.38688612</v>
       </c>
       <c r="K15" s="7">
         <f ca="1">IF(K2&gt;Measles!B11,Measles!B11,IF(Scenario_data!K2 &lt;Measles!A11,Measles!A11,Scenario_data!K2))</f>
-        <v>699194982.27341413</v>
+        <v>1054136692.0376759</v>
       </c>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
@@ -3667,43 +3667,43 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(B3&gt;Mumps!B2,Mumps!B2,IF(Scenario_data!B3 &lt;Mumps!A2,Mumps!A2,Scenario_data!B3))</f>
-        <v>29353628.074818686</v>
+        <v>20840110.913639396</v>
       </c>
       <c r="C16" s="7">
         <f ca="1">IF(C3&gt;Mumps!B3,Mumps!B3,IF(Scenario_data!C3 &lt;Mumps!A3,Mumps!A3,Scenario_data!C3))</f>
-        <v>32537650.044107866</v>
+        <v>33003198.189924993</v>
       </c>
       <c r="D16" s="7">
         <f ca="1">IF(D3&gt;Mumps!B4,Mumps!B4,IF(Scenario_data!D3 &lt;Mumps!A4,Mumps!A4,Scenario_data!D3))</f>
-        <v>39366857.745121069</v>
+        <v>37564948.897706904</v>
       </c>
       <c r="E16" s="7">
         <f ca="1">IF(E3&gt;Mumps!B5,Mumps!B5,IF(Scenario_data!E3 &lt;Mumps!A5,Mumps!A5,Scenario_data!E3))</f>
-        <v>34343404.950566143</v>
+        <v>38297819.090270177</v>
       </c>
       <c r="F16" s="7">
         <f ca="1">IF(F3&gt;Mumps!B6,Mumps!B6,IF(Scenario_data!F3 &lt;Mumps!A6,Mumps!A6,Scenario_data!F3))</f>
-        <v>46741141.994529955</v>
+        <v>43196820.504247271</v>
       </c>
       <c r="G16" s="7">
         <f ca="1">IF(G3&gt;Mumps!B7,Mumps!B7,IF(Scenario_data!G3 &lt;Mumps!A7,Mumps!A7,Scenario_data!G3))</f>
-        <v>31092524.433205169</v>
+        <v>40800099.727116153</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">IF(H3&gt;Mumps!B8,Mumps!B8,IF(Scenario_data!H3 &lt;Mumps!A8,Mumps!A8,Scenario_data!H3))</f>
-        <v>59019489.163654804</v>
+        <v>55512117.873587593</v>
       </c>
       <c r="I16" s="7">
         <f ca="1">IF(I3&gt;Mumps!B9,Mumps!B9,IF(Scenario_data!I3 &lt;Mumps!A9,Mumps!A9,Scenario_data!I3))</f>
-        <v>54156045.118848495</v>
+        <v>42130742.493162677</v>
       </c>
       <c r="J16" s="7">
         <f ca="1">IF(J3&gt;Mumps!B10,Mumps!B10,IF(Scenario_data!J3 &lt;Mumps!A10,Mumps!A10,Scenario_data!J3))</f>
-        <v>48931800.745717496</v>
+        <v>51577977.658602305</v>
       </c>
       <c r="K16" s="7">
         <f ca="1">IF(K3&gt;Mumps!B11,Mumps!B11,IF(Scenario_data!K3 &lt;Mumps!A11,Mumps!A11,Scenario_data!K3))</f>
-        <v>70878049.684350103</v>
+        <v>62584548.099562094</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -3712,43 +3712,43 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(B4&gt;Rubella!B2,Rubella!B2,IF(Scenario_data!B4 &lt;Rubella!A2,Rubella!A2,Scenario_data!B4))</f>
-        <v>408745810.96556836</v>
+        <v>272373463.40747488</v>
       </c>
       <c r="C17" s="7">
         <f ca="1">IF(C4&gt;Rubella!B3,Rubella!B3,IF(Scenario_data!C4 &lt;Rubella!A3,Rubella!A3,Scenario_data!C4))</f>
-        <v>424609749.97643918</v>
+        <v>483516328.73493004</v>
       </c>
       <c r="D17" s="7">
         <f ca="1">IF(D4&gt;Rubella!B4,Rubella!B4,IF(Scenario_data!D4 &lt;Rubella!A4,Rubella!A4,Scenario_data!D4))</f>
-        <v>421344487.24847007</v>
+        <v>289119898.10361594</v>
       </c>
       <c r="E17" s="7">
         <f ca="1">IF(E4&gt;Rubella!B5,Rubella!B5,IF(Scenario_data!E4 &lt;Rubella!A5,Rubella!A5,Scenario_data!E4))</f>
-        <v>486789456.52070808</v>
+        <v>414059893.41429448</v>
       </c>
       <c r="F17" s="7">
         <f ca="1">IF(F4&gt;Rubella!B6,Rubella!B6,IF(Scenario_data!F4 &lt;Rubella!A6,Rubella!A6,Scenario_data!F4))</f>
-        <v>533594749.31181866</v>
+        <v>432718696.23840481</v>
       </c>
       <c r="G17" s="7">
         <f ca="1">IF(G4&gt;Rubella!B7,Rubella!B7,IF(Scenario_data!G4 &lt;Rubella!A7,Rubella!A7,Scenario_data!G4))</f>
-        <v>516430997.50526792</v>
+        <v>648180888.19893277</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">IF(H4&gt;Rubella!B8,Rubella!B8,IF(Scenario_data!H4 &lt;Rubella!A8,Rubella!A8,Scenario_data!H4))</f>
-        <v>854302314.37320733</v>
+        <v>734672167.46613932</v>
       </c>
       <c r="I17" s="7">
         <f ca="1">IF(I4&gt;Rubella!B9,Rubella!B9,IF(Scenario_data!I4 &lt;Rubella!A9,Rubella!A9,Scenario_data!I4))</f>
-        <v>727522986.83084035</v>
+        <v>821487018.30194342</v>
       </c>
       <c r="J17" s="7">
         <f ca="1">IF(J4&gt;Rubella!B10,Rubella!B10,IF(Scenario_data!J4 &lt;Rubella!A10,Rubella!A10,Scenario_data!J4))</f>
-        <v>813449257.77919173</v>
+        <v>817668241.94867456</v>
       </c>
       <c r="K17" s="7">
         <f ca="1">IF(K4&gt;Rubella!B12=1,Rubella!B11,IF(Scenario_data!K4 &lt;Rubella!A11,Rubella!A11,Scenario_data!K4))</f>
-        <v>799136936.70137048</v>
+        <v>695484711.98491108</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -3757,43 +3757,43 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(B5&gt;Diphtheria!B2,Diphtheria!B2,IF(Scenario_data!B5 &lt;Diphtheria!A2,Diphtheria!A2,Scenario_data!B5))</f>
-        <v>625302065.02012849</v>
+        <v>652096368.2216897</v>
       </c>
       <c r="C18" s="7">
         <f ca="1">IF(C5&gt;Diphtheria!B3,Diphtheria!B3,IF(Scenario_data!C5 &lt;Diphtheria!A3,Diphtheria!A3,Scenario_data!C5))</f>
-        <v>706692052.3953979</v>
+        <v>674341526.85532749</v>
       </c>
       <c r="D18" s="7">
         <f ca="1">IF(D5&gt;Diphtheria!B4,Diphtheria!B4,IF(Scenario_data!D5 &lt;Diphtheria!A4,Diphtheria!A4,Scenario_data!D5))</f>
-        <v>750543450.11648631</v>
+        <v>717706771.55113971</v>
       </c>
       <c r="E18" s="7">
         <f ca="1">IF(E5&gt;Diphtheria!B5,Diphtheria!B5,IF(Scenario_data!E5 &lt;Diphtheria!A5,Diphtheria!A5,Scenario_data!E5))</f>
-        <v>816565360.60382926</v>
+        <v>934898423.3402555</v>
       </c>
       <c r="F18" s="7">
         <f ca="1">IF(F5&gt;Diphtheria!B6,Diphtheria!B6,IF(Scenario_data!F5 &lt;Diphtheria!A6,Diphtheria!A6,Scenario_data!F5))</f>
-        <v>970683647.47504902</v>
+        <v>910992813.42327571</v>
       </c>
       <c r="G18" s="7">
         <f ca="1">IF(G5&gt;Diphtheria!B7,Diphtheria!B7,IF(Scenario_data!G5 &lt;Diphtheria!A7,Diphtheria!A7,Scenario_data!G5))</f>
-        <v>1208008489.5923297</v>
+        <v>1182799454.738198</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">IF(H5&gt;Diphtheria!B8,Diphtheria!B8,IF(Scenario_data!H5 &lt;Diphtheria!A8,Diphtheria!A8,Scenario_data!H5))</f>
-        <v>1352307677.5593073</v>
+        <v>1384125950.1142042</v>
       </c>
       <c r="I18" s="7">
         <f ca="1">IF(I5&gt;Diphtheria!B9,Diphtheria!B9,IF(Scenario_data!I5 &lt;Diphtheria!A9,Diphtheria!A9,Scenario_data!I5))</f>
-        <v>1617517085.2339122</v>
+        <v>1604956477.0636852</v>
       </c>
       <c r="J18" s="7">
         <f ca="1">IF(J5&gt;Diphtheria!B10,Diphtheria!B10,IF(Scenario_data!J5 &lt;Diphtheria!A10,Diphtheria!A10,Scenario_data!J5))</f>
-        <v>1625663109.9002686</v>
+        <v>1648666503.6256371</v>
       </c>
       <c r="K18" s="7">
         <f ca="1">IF(K5&gt;Diphtheria!B11,Diphtheria!B11,IF(Scenario_data!K5 &lt;Diphtheria!A11,Diphtheria!A11,Scenario_data!K5))</f>
-        <v>1902813642.1379783</v>
+        <v>2003485736.807965</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -3802,43 +3802,43 @@
       </c>
       <c r="B19" s="7">
         <f ca="1">IF(B6&gt;Tetanus!B2,Tetanus!B2,IF(Scenario_data!B6 &lt;Tetanus!A2,Tetanus!A2,Scenario_data!B6))</f>
-        <v>650970822.56898654</v>
+        <v>580321768.84763432</v>
       </c>
       <c r="C19" s="7">
         <f ca="1">IF(C6&gt;Tetanus!B3,Tetanus!B3,IF(Scenario_data!C6 &lt;Tetanus!A3,Tetanus!A3,Scenario_data!C6))</f>
-        <v>619268075.03400934</v>
+        <v>618409157.36515844</v>
       </c>
       <c r="D19" s="7">
         <f ca="1">IF(D6&gt;Tetanus!B4,Tetanus!B4,IF(Scenario_data!D6 &lt;Tetanus!A4,Tetanus!A4,Scenario_data!D6))</f>
-        <v>631788067.9471004</v>
+        <v>646864171.13713646</v>
       </c>
       <c r="E19" s="7">
         <f ca="1">IF(E6&gt;Tetanus!B5,Tetanus!B5,IF(Scenario_data!E6 &lt;Tetanus!A5,Tetanus!A5,Scenario_data!E6))</f>
-        <v>691384012.4254334</v>
+        <v>675476437.66133559</v>
       </c>
       <c r="F19" s="7">
         <f ca="1">IF(F6&gt;Tetanus!B6,Tetanus!B6,IF(Scenario_data!F6 &lt;Tetanus!A6,Tetanus!A6,Scenario_data!F6))</f>
-        <v>675440352.04472125</v>
+        <v>707358024.11453915</v>
       </c>
       <c r="G19" s="7">
         <f ca="1">IF(G6&gt;Tetanus!B7,Tetanus!B7,IF(Scenario_data!G6 &lt;Tetanus!A7,Tetanus!A7,Scenario_data!G6))</f>
-        <v>701056726.73188722</v>
+        <v>705923805.05312788</v>
       </c>
       <c r="H19" s="7">
         <f ca="1">IF(H6&gt;Tetanus!B8,Tetanus!B8,IF(Scenario_data!H6 &lt;Tetanus!A8,Tetanus!A8,Scenario_data!H6))</f>
-        <v>676359138.52133548</v>
+        <v>677684598.1991353</v>
       </c>
       <c r="I19" s="7">
         <f ca="1">IF(I6&gt;Tetanus!B9,Tetanus!B9,IF(Scenario_data!I6 &lt;Tetanus!A9,Tetanus!A9,Scenario_data!I6))</f>
-        <v>704159366.74474478</v>
+        <v>756577838.53838158</v>
       </c>
       <c r="J19" s="7">
         <f ca="1">IF(J6&gt;Tetanus!B10,Tetanus!B10,IF(Scenario_data!J6 &lt;Tetanus!A10,Tetanus!A10,Scenario_data!J6))</f>
-        <v>706345126.76525784</v>
+        <v>712522135.88390744</v>
       </c>
       <c r="K19" s="7">
         <f ca="1">IF(K6&gt;Tetanus!B11,Tetanus!B11,IF(Scenario_data!K6 &lt;Tetanus!A11,Tetanus!A11,Scenario_data!K6))</f>
-        <v>722315359.08481681</v>
+        <v>744577945.9480027</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -3847,43 +3847,43 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IF(B7&gt;Pertussis!B2,Pertussis!B2,IF(Scenario_data!B7 &lt;Pertussis!A2,Pertussis!A2,Scenario_data!B7))</f>
-        <v>369019997.25248706</v>
+        <v>377099079.522255</v>
       </c>
       <c r="C20" s="7">
         <f ca="1">IF(C7&gt;Pertussis!B3,Pertussis!B3,IF(Scenario_data!C7 &lt;Pertussis!A3,Pertussis!A3,Scenario_data!C7))</f>
-        <v>327075398.68409991</v>
+        <v>349743008.42086285</v>
       </c>
       <c r="D20" s="7">
         <f ca="1">IF(D7&gt;Pertussis!B4,Pertussis!B4,IF(Scenario_data!D7 &lt;Pertussis!A4,Pertussis!A4,Scenario_data!D7))</f>
-        <v>329416556.92000383</v>
+        <v>358828924.65739149</v>
       </c>
       <c r="E20" s="7">
         <f ca="1">IF(E7&gt;Pertussis!B5,Pertussis!B5,IF(Scenario_data!E7 &lt;Pertussis!A5,Pertussis!A5,Scenario_data!E7))</f>
-        <v>360936826.88394058</v>
+        <v>384166685.06519914</v>
       </c>
       <c r="F20" s="7">
         <f ca="1">IF(F7&gt;Pertussis!B6,Pertussis!B6,IF(Scenario_data!F7 &lt;Pertussis!A6,Pertussis!A6,Scenario_data!F7))</f>
-        <v>379958217.69572496</v>
+        <v>321018131.2935856</v>
       </c>
       <c r="G20" s="7">
         <f ca="1">IF(G7&gt;Pertussis!B7,Pertussis!B7,IF(Scenario_data!G7 &lt;Pertussis!A7,Pertussis!A7,Scenario_data!G7))</f>
-        <v>322281409.03089046</v>
+        <v>371783799.60341054</v>
       </c>
       <c r="H20" s="7">
         <f ca="1">IF(H7&gt;Pertussis!B8,Pertussis!B8,IF(Scenario_data!H7 &lt;Pertussis!A8,Pertussis!A8,Scenario_data!H7))</f>
-        <v>402541327.16018939</v>
+        <v>361224164.75770944</v>
       </c>
       <c r="I20" s="7">
         <f ca="1">IF(I7&gt;Pertussis!B9,Pertussis!B9,IF(Scenario_data!I7 &lt;Pertussis!A9,Pertussis!A9,Scenario_data!I7))</f>
-        <v>359028892.43529868</v>
+        <v>379838866.49923599</v>
       </c>
       <c r="J20" s="7">
         <f ca="1">IF(J7&gt;Pertussis!B10,Pertussis!B10,IF(Scenario_data!J7 &lt;Pertussis!A10,Pertussis!A10,Scenario_data!J7))</f>
-        <v>325242719.89408427</v>
+        <v>397507726.06506461</v>
       </c>
       <c r="K20" s="7">
         <f ca="1">IF(K7&gt;Pertussis!B11,Pertussis!B11,IF(Scenario_data!K7 &lt;Pertussis!A11,Pertussis!A11,Scenario_data!K7))</f>
-        <v>421465050.10378128</v>
+        <v>400664505.44185388</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -3892,43 +3892,43 @@
       </c>
       <c r="B21" s="7">
         <f ca="1">IF(B8&gt;Hepatitis_B!B2,Hepatitis_B!B2,IF(Scenario_data!B8 &lt;Hepatitis_B!A2,Hepatitis_B!A2,Scenario_data!B8))</f>
-        <v>355778692.35009098</v>
+        <v>390859091.0957067</v>
       </c>
       <c r="C21" s="7">
         <f ca="1">IF(C8&gt;Hepatitis_B!B3,Hepatitis_B!B3,IF(Scenario_data!C8 &lt;Hepatitis_B!A3,Hepatitis_B!A3,Scenario_data!C8))</f>
-        <v>438002523.10604686</v>
+        <v>385955632.35852683</v>
       </c>
       <c r="D21" s="7">
         <f ca="1">IF(D8&gt;Hepatitis_B!B4,Hepatitis_B!B4,IF(Scenario_data!D8 &lt;Hepatitis_B!A4,Hepatitis_B!A4,Scenario_data!D8))</f>
-        <v>389734412.31942236</v>
+        <v>323629206.30780774</v>
       </c>
       <c r="E21" s="7">
         <f ca="1">IF(E8&gt;Hepatitis_B!B5,Hepatitis_B!B5,IF(Scenario_data!E8 &lt;Hepatitis_B!A5,Hepatitis_B!A5,Scenario_data!E8))</f>
-        <v>403817107.07063323</v>
+        <v>424663649.35197407</v>
       </c>
       <c r="F21" s="7">
         <f ca="1">IF(F8&gt;Hepatitis_B!B6,Hepatitis_B!B6,IF(Scenario_data!F8 &lt;Hepatitis_B!A6,Hepatitis_B!A6,Scenario_data!F8))</f>
-        <v>391327351.94039482</v>
+        <v>373482318.40589166</v>
       </c>
       <c r="G21" s="7">
         <f ca="1">IF(G8&gt;Hepatitis_B!B7,Hepatitis_B!B7,IF(Scenario_data!G8 &lt;Hepatitis_B!A7,Hepatitis_B!A7,Scenario_data!G8))</f>
-        <v>452020208.05661857</v>
+        <v>358036029.12115455</v>
       </c>
       <c r="H21" s="7">
         <f ca="1">IF(H8&gt;Hepatitis_B!B8,Hepatitis_B!B8,IF(Scenario_data!H8 &lt;Hepatitis_B!A8,Hepatitis_B!A8,Scenario_data!H8))</f>
-        <v>361744045.68037063</v>
+        <v>480866833.4064604</v>
       </c>
       <c r="I21" s="7">
         <f ca="1">IF(I8&gt;Hepatitis_B!B9,Hepatitis_B!B9,IF(Scenario_data!I8 &lt;Hepatitis_B!A9,Hepatitis_B!A9,Scenario_data!I8))</f>
-        <v>373964982.33362991</v>
+        <v>476777441.9324975</v>
       </c>
       <c r="J21" s="7">
         <f ca="1">IF(J8&gt;Hepatitis_B!B10,Hepatitis_B!B10,IF(Scenario_data!J8 &lt;Hepatitis_B!A10,Hepatitis_B!A10,Scenario_data!J8))</f>
-        <v>427884781.59073621</v>
+        <v>438033992.66444403</v>
       </c>
       <c r="K21" s="7">
         <f ca="1">IF(K8&gt;Hepatitis_B!B11,Hepatitis_B!B11,IF(Scenario_data!K8 &lt;Hepatitis_B!A11,Hepatitis_B!A11,Scenario_data!K8))</f>
-        <v>436086533.40796435</v>
+        <v>424575883.86303997</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -3937,43 +3937,43 @@
       </c>
       <c r="B22" s="7">
         <f ca="1">IF(B9&gt;Hib!B2,Hib!B2,IF(Scenario_data!B9 &lt;Hib!A2,Hib!A2,Scenario_data!B9))</f>
-        <v>289359717.07491219</v>
+        <v>300732688.74825186</v>
       </c>
       <c r="C22" s="7">
         <f ca="1">IF(C9&gt;Hib!B3,Hib!B3,IF(Scenario_data!C9 &lt;Hib!A3,Hib!A3,Scenario_data!C9))</f>
-        <v>313363487.12721384</v>
+        <v>301138426.85186619</v>
       </c>
       <c r="D22" s="7">
         <f ca="1">IF(D9&gt;Hib!B4,Hib!B4,IF(Scenario_data!D9 &lt;Hib!A4,Hib!A4,Scenario_data!D9))</f>
-        <v>343475515.11765915</v>
+        <v>352704690.37444395</v>
       </c>
       <c r="E22" s="7">
         <f ca="1">IF(E9&gt;Hib!B5,Hib!B5,IF(Scenario_data!E9 &lt;Hib!A5,Hib!A5,Scenario_data!E9))</f>
-        <v>334837340.45689988</v>
+        <v>346461019.72448152</v>
       </c>
       <c r="F22" s="7">
         <f ca="1">IF(F9&gt;Hib!B6,Hib!B6,IF(Scenario_data!F9 &lt;Hib!A6,Hib!A6,Scenario_data!F9))</f>
-        <v>363884818.47186959</v>
+        <v>357200804.05163914</v>
       </c>
       <c r="G22" s="7">
         <f ca="1">IF(G9&gt;Hib!B7,Hib!B7,IF(Scenario_data!G9 &lt;Hib!A7,Hib!A7,Scenario_data!G9))</f>
-        <v>357188006.89770454</v>
+        <v>312268189.61223459</v>
       </c>
       <c r="H22" s="7">
         <f ca="1">IF(H9&gt;Hib!B8,Hib!B8,IF(Scenario_data!H9 &lt;Hib!A8,Hib!A8,Scenario_data!H9))</f>
-        <v>348934285.05260718</v>
+        <v>360212222.90886766</v>
       </c>
       <c r="I22" s="7">
         <f ca="1">IF(I9&gt;Hib!B9,Hib!B9,IF(Scenario_data!I9 &lt;Hib!A9,Hib!A9,Scenario_data!I9))</f>
-        <v>381549183.42356211</v>
+        <v>375709755.60838896</v>
       </c>
       <c r="J22" s="7">
         <f ca="1">IF(J9&gt;Hib!B10,Hib!B10,IF(Scenario_data!J9 &lt;Hib!A10,Hib!A10,Scenario_data!J9))</f>
-        <v>409555583.44038814</v>
+        <v>397730594.11381888</v>
       </c>
       <c r="K22" s="7">
         <f ca="1">IF(K9&gt;Hib!B11,Hib!B11,IF(Scenario_data!K9 &lt;Hib!A11,Hib!A11,Scenario_data!K9))</f>
-        <v>403900578.3239277</v>
+        <v>425669766.29332536</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -3982,43 +3982,43 @@
       </c>
       <c r="B23" s="7">
         <f ca="1">IF(B10&gt;Polio!B2,Polio!B2,IF(Scenario_data!B10 &lt;Polio!A2,Polio!A2,Scenario_data!B10))</f>
-        <v>581839336.02645445</v>
+        <v>587059615.91624844</v>
       </c>
       <c r="C23" s="7">
         <f ca="1">IF(C10&gt;Polio!B3,Polio!B3,IF(Scenario_data!C10 &lt;Polio!A3,Polio!A3,Scenario_data!C10))</f>
-        <v>649172550.55085421</v>
+        <v>711589396.21656442</v>
       </c>
       <c r="D23" s="7">
         <f ca="1">IF(D10&gt;Polio!B4,Polio!B4,IF(Scenario_data!D10 &lt;Polio!A4,Polio!A4,Scenario_data!D10))</f>
-        <v>567159776.66132641</v>
+        <v>695287580.72666001</v>
       </c>
       <c r="E23" s="7">
         <f ca="1">IF(E10&gt;Polio!B5,Polio!B5,IF(Scenario_data!E10 &lt;Polio!A5,Polio!A5,Scenario_data!E10))</f>
-        <v>692694739.33496797</v>
+        <v>768463061.4913609</v>
       </c>
       <c r="F23" s="7">
         <f ca="1">IF(F10&gt;Polio!B6,Polio!B6,IF(Scenario_data!F10 &lt;Polio!A6,Polio!A6,Scenario_data!F10))</f>
-        <v>717832136.94679999</v>
+        <v>718238764.86178637</v>
       </c>
       <c r="G23" s="7">
         <f ca="1">IF(G10&gt;Polio!B7,Polio!B7,IF(Scenario_data!G10 &lt;Polio!A7,Polio!A7,Scenario_data!G10))</f>
-        <v>834927990.10967553</v>
+        <v>753604437.83078837</v>
       </c>
       <c r="H23" s="7">
         <f ca="1">IF(H10&gt;Polio!B8,Polio!B8,IF(Scenario_data!H10 &lt;Polio!A8,Polio!A8,Scenario_data!H10))</f>
-        <v>803843472.5752368</v>
+        <v>839210342.65936148</v>
       </c>
       <c r="I23" s="7">
         <f ca="1">IF(I10&gt;Polio!B9,Polio!B9,IF(Scenario_data!I10 &lt;Polio!A9,Polio!A9,Scenario_data!I10))</f>
-        <v>797130260.47852981</v>
+        <v>804551762.56089425</v>
       </c>
       <c r="J23" s="7">
         <f ca="1">IF(J10&gt;Polio!B10,Polio!B10,IF(Scenario_data!J10 &lt;Polio!A10,Polio!A10,Scenario_data!J10))</f>
-        <v>830331997.11825132</v>
+        <v>881493869.87954855</v>
       </c>
       <c r="K23" s="7">
         <f ca="1">IF(K10&gt;Polio!B11,Polio!B11,IF(Scenario_data!K10 &lt;Polio!A11,Polio!A11,Scenario_data!K10))</f>
-        <v>954723224.3480581</v>
+        <v>859201436.88993907</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -4027,43 +4027,43 @@
       </c>
       <c r="B24" s="7">
         <f ca="1">IF(B11&gt;HPV!B2,HPV!B2,IF(Scenario_data!B11 &lt;HPV!A2,HPV!A2,Scenario_data!B11))</f>
-        <v>28813061.981344361</v>
+        <v>27250263.793651372</v>
       </c>
       <c r="C24" s="7">
         <f ca="1">IF(C11&gt;HPV!B3,HPV!B3,IF(Scenario_data!C11 &lt;HPV!A3,HPV!A3,Scenario_data!C11))</f>
-        <v>34513806.317383148</v>
+        <v>33604048.931154117</v>
       </c>
       <c r="D24" s="7">
         <f ca="1">IF(D11&gt;HPV!B4,HPV!B4,IF(Scenario_data!D11 &lt;HPV!A4,HPV!A4,Scenario_data!D11))</f>
-        <v>40246926.621811047</v>
+        <v>42521002.697570607</v>
       </c>
       <c r="E24" s="7">
         <f ca="1">IF(E11&gt;HPV!B5,HPV!B5,IF(Scenario_data!E11 &lt;HPV!A5,HPV!A5,Scenario_data!E11))</f>
-        <v>45395490.20459792</v>
+        <v>46309572.189586237</v>
       </c>
       <c r="F24" s="7">
         <f ca="1">IF(F11&gt;HPV!B6,HPV!B6,IF(Scenario_data!F11 &lt;HPV!A6,HPV!A6,Scenario_data!F11))</f>
-        <v>56830506.861267693</v>
+        <v>55327907.464503817</v>
       </c>
       <c r="G24" s="7">
         <f ca="1">IF(G11&gt;HPV!B7,HPV!B7,IF(Scenario_data!G11 &lt;HPV!A7,HPV!A7,Scenario_data!G11))</f>
-        <v>59228362.113960996</v>
+        <v>59490904.512177654</v>
       </c>
       <c r="H24" s="7">
         <f ca="1">IF(H11&gt;HPV!B8,HPV!B8,IF(Scenario_data!H11 &lt;HPV!A8,HPV!A8,Scenario_data!H11))</f>
-        <v>67963050.336423963</v>
+        <v>65506111.644410707</v>
       </c>
       <c r="I24" s="7">
         <f ca="1">IF(I11&gt;HPV!B9,HPV!B9,IF(Scenario_data!I11 &lt;HPV!A9,HPV!A9,Scenario_data!I11))</f>
-        <v>73398426.17083995</v>
+        <v>71881059.651827395</v>
       </c>
       <c r="J24" s="7">
         <f ca="1">IF(J11&gt;HPV!B10,HPV!B10,IF(Scenario_data!J11 &lt;HPV!A10,HPV!A10,Scenario_data!J11))</f>
-        <v>83823211.643525869</v>
+        <v>79714888.524668857</v>
       </c>
       <c r="K24" s="7">
         <f ca="1">IF(K11&gt;HPV!B11,HPV!B11,IF(Scenario_data!K11 &lt;HPV!A11,HPV!A11,Scenario_data!K11))</f>
-        <v>89659414.119553238</v>
+        <v>87510069.202634826</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -4072,43 +4072,43 @@
       </c>
       <c r="B25" s="7">
         <f ca="1">IF(B12&gt;Rotavirus!B2,Rotavirus!B2,IF(Scenario_data!B12 &lt;Rotavirus!A2,Rotavirus!A2,Scenario_data!B12))</f>
-        <v>212356179.18269354</v>
+        <v>203184261.34051713</v>
       </c>
       <c r="C25" s="7">
         <f ca="1">IF(C12&gt;Rotavirus!B3,Rotavirus!B3,IF(Scenario_data!C12 &lt;Rotavirus!A3,Rotavirus!A3,Scenario_data!C12))</f>
-        <v>228002743.31291083</v>
+        <v>193888232.76516005</v>
       </c>
       <c r="D25" s="7">
         <f ca="1">IF(D12&gt;Rotavirus!B4,Rotavirus!B4,IF(Scenario_data!D12 &lt;Rotavirus!A4,Rotavirus!A4,Scenario_data!D12))</f>
-        <v>226863050.68823063</v>
+        <v>237913229.93208605</v>
       </c>
       <c r="E25" s="7">
         <f ca="1">IF(E12&gt;Rotavirus!B5,Rotavirus!B5,IF(Scenario_data!E12 &lt;Rotavirus!A5,Rotavirus!A5,Scenario_data!E12))</f>
-        <v>299343945.00113678</v>
+        <v>244389697.47415298</v>
       </c>
       <c r="F25" s="7">
         <f ca="1">IF(F12&gt;Rotavirus!B6,Rotavirus!B6,IF(Scenario_data!F12 &lt;Rotavirus!A6,Rotavirus!A6,Scenario_data!F12))</f>
-        <v>316684901.98480678</v>
+        <v>349629111.22157079</v>
       </c>
       <c r="G25" s="7">
         <f ca="1">IF(G12&gt;Rotavirus!B7,Rotavirus!B7,IF(Scenario_data!G12 &lt;Rotavirus!A7,Rotavirus!A7,Scenario_data!G12))</f>
-        <v>372084322.09227526</v>
+        <v>427250110.0740537</v>
       </c>
       <c r="H25" s="7">
         <f ca="1">IF(H12&gt;Rotavirus!B8,Rotavirus!B8,IF(Scenario_data!H12 &lt;Rotavirus!A8,Rotavirus!A8,Scenario_data!H12))</f>
-        <v>447559080.14459324</v>
+        <v>457142117.25461364</v>
       </c>
       <c r="I25" s="7">
         <f ca="1">IF(I12&gt;Rotavirus!B9,Rotavirus!B9,IF(Scenario_data!I12 &lt;Rotavirus!A9,Rotavirus!A9,Scenario_data!I12))</f>
-        <v>524263673.48202568</v>
+        <v>507144865.37986726</v>
       </c>
       <c r="J25" s="7">
         <f ca="1">IF(J12&gt;Rotavirus!B10,Rotavirus!B10,IF(Scenario_data!J12 &lt;Rotavirus!A10,Rotavirus!A10,Scenario_data!J12))</f>
-        <v>600000823.35737109</v>
+        <v>647901558.97098541</v>
       </c>
       <c r="K25" s="7">
         <f ca="1">IF(K12&gt;Rotavirus!B11,Rotavirus!B11,IF(Scenario_data!K12 &lt;Rotavirus!A11,Rotavirus!A11,Scenario_data!K12))</f>
-        <v>743326072.76503897</v>
+        <v>737219212.85431552</v>
       </c>
       <c r="M25" s="4"/>
     </row>
@@ -4118,43 +4118,43 @@
       </c>
       <c r="B26" s="7">
         <f ca="1">IF(B13&gt;PCV!B2,PCV!B2,IF(Scenario_data!B13 &lt;PCV!A2,PCV!A2,Scenario_data!B13))</f>
-        <v>234292637.76584065</v>
+        <v>211403260.01881739</v>
       </c>
       <c r="C26" s="7">
         <f ca="1">IF(C13&gt;PCV!B3,PCV!B3,IF(Scenario_data!C13 &lt;PCV!A3,PCV!A3,Scenario_data!C13))</f>
-        <v>251340614.35331798</v>
+        <v>251439115.74413413</v>
       </c>
       <c r="D26" s="7">
         <f ca="1">IF(D13&gt;PCV!B4,PCV!B4,IF(Scenario_data!D13 &lt;PCV!A4,PCV!A4,Scenario_data!D13))</f>
-        <v>286798993.08894235</v>
+        <v>270272253.56533325</v>
       </c>
       <c r="E26" s="7">
         <f ca="1">IF(E13&gt;PCV!B5,PCV!B5,IF(Scenario_data!E13 &lt;PCV!A5,PCV!A5,Scenario_data!E13))</f>
-        <v>318702438.85792321</v>
+        <v>317723220.10685098</v>
       </c>
       <c r="F26" s="7">
         <f ca="1">IF(F13&gt;PCV!B6,PCV!B6,IF(Scenario_data!F13 &lt;PCV!A6,PCV!A6,Scenario_data!F13))</f>
-        <v>337336416.02681231</v>
+        <v>337170221.39178747</v>
       </c>
       <c r="G26" s="7">
         <f ca="1">IF(G13&gt;PCV!B7,PCV!B7,IF(Scenario_data!G13 &lt;PCV!A7,PCV!A7,Scenario_data!G13))</f>
-        <v>368705685.98718059</v>
+        <v>365214546.95532507</v>
       </c>
       <c r="H26" s="7">
         <f ca="1">IF(H13&gt;PCV!B8,PCV!B8,IF(Scenario_data!H13 &lt;PCV!A8,PCV!A8,Scenario_data!H13))</f>
-        <v>408722386.12393236</v>
+        <v>395976114.41627443</v>
       </c>
       <c r="I26" s="7">
         <f ca="1">IF(I13&gt;PCV!B9,PCV!B9,IF(Scenario_data!I13 &lt;PCV!A9,PCV!A9,Scenario_data!I13))</f>
-        <v>451798991.30340707</v>
+        <v>449048557.10372937</v>
       </c>
       <c r="J26" s="7">
         <f ca="1">IF(J13&gt;PCV!B10,PCV!B10,IF(Scenario_data!J13 &lt;PCV!A10,PCV!A10,Scenario_data!J13))</f>
-        <v>478974333.83229929</v>
+        <v>495827019.50174165</v>
       </c>
       <c r="K26" s="7">
         <f ca="1">IF(K13&gt;PCV!B11,PCV!B11,IF(Scenario_data!K13 &lt;PCV!A11,PCV!A11,Scenario_data!K13))</f>
-        <v>425893971.36649722</v>
+        <v>418569031.30105716</v>
       </c>
       <c r="M26" s="4"/>
     </row>

</xml_diff>

<commit_message>
added model notation documents; working on discounts
</commit_message>
<xml_diff>
--- a/DATA/demand/antigen_CI_Random_generator.xlsx
+++ b/DATA/demand/antigen_CI_Random_generator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/demand/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="600" documentId="11_4A5645C871AEA98286DE389EAFF8EF0F542BC54D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27C78165-C171-4D6F-B0EC-D41AEC39E222}"/>
+  <xr:revisionPtr revIDLastSave="603" documentId="11_4A5645C871AEA98286DE389EAFF8EF0F542BC54D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74B5E9CD-00B0-4057-8956-E930C6C7739A}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-7070" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Diphtheria" sheetId="1" r:id="rId1"/>
@@ -336,34 +336,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>380279116.3628819</c:v>
+                  <c:v>427844524.08335775</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>448989663.26277512</c:v>
+                  <c:v>266493540.45622987</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>579693559.67794991</c:v>
+                  <c:v>690921430.33690572</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>477216801.40458322</c:v>
+                  <c:v>608559229.60524082</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>524049735.38377869</c:v>
+                  <c:v>663849922.05193794</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>786493791.26628435</c:v>
+                  <c:v>720017052.81562459</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>792703264.83761966</c:v>
+                  <c:v>889418994.55034482</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>837398630.38757217</c:v>
+                  <c:v>904042059.50542402</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1002521692.9763725</c:v>
+                  <c:v>1015447126.9340428</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1042180640.7550312</c:v>
+                  <c:v>924995113.19309568</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -408,34 +408,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>32802801.1819687</c:v>
+                  <c:v>32215325.210729256</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>32297080.572214447</c:v>
+                  <c:v>45516332.979260825</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>36664014.975054443</c:v>
+                  <c:v>33898087.031309105</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>35606772.83373329</c:v>
+                  <c:v>42814676.437276535</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28353686.142964706</c:v>
+                  <c:v>36449281.749024712</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>46353460.324733652</c:v>
+                  <c:v>34376475.810845077</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>47386539.516075164</c:v>
+                  <c:v>39757843.010042816</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>48049849.411365598</c:v>
+                  <c:v>49608710.232102938</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>57006990.622826666</c:v>
+                  <c:v>64076046.965096839</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>71338965.681571722</c:v>
+                  <c:v>53151222.967799768</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -480,34 +480,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>455737876.75224012</c:v>
+                  <c:v>321465048.4790833</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>279191668.70165825</c:v>
+                  <c:v>338050229.20354372</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>491718464.82244426</c:v>
+                  <c:v>383103937.96252614</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>321478288.58388901</c:v>
+                  <c:v>566246441.65829504</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>582569187.24174964</c:v>
+                  <c:v>462931671.903368</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>676324219.36442959</c:v>
+                  <c:v>678288191.2504704</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>707046972.46634114</c:v>
+                  <c:v>685059803.96362448</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>696541735.38053691</c:v>
+                  <c:v>481911360.12481743</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>729825228.35502946</c:v>
+                  <c:v>628165183.97071981</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>912144063.31862998</c:v>
+                  <c:v>706453621.3172642</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -552,34 +552,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>730027462.43859041</c:v>
+                  <c:v>625306808.80609596</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>748870069.02099586</c:v>
+                  <c:v>574773030.64024889</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>857570894.05129778</c:v>
+                  <c:v>723594153.53824306</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>841796851.68876898</c:v>
+                  <c:v>840827455.21154118</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>940427660.20165586</c:v>
+                  <c:v>839566408.24645913</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>997410651.78942442</c:v>
+                  <c:v>1175682702.2142451</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1342376979.3438168</c:v>
+                  <c:v>1345041665.9302816</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1609134848.1879845</c:v>
+                  <c:v>1635771765.4634292</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1583518014.6048779</c:v>
+                  <c:v>1608781146.4265878</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1863693054.9682305</c:v>
+                  <c:v>1925303189.7746534</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -624,34 +624,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>665645372.21190369</c:v>
+                  <c:v>638898240.21864259</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>635600563.96215916</c:v>
+                  <c:v>645057838.57984638</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>726256426.06573796</c:v>
+                  <c:v>635282685.42925298</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>709842146.89628315</c:v>
+                  <c:v>699956110.31624317</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>678579538.7353512</c:v>
+                  <c:v>709104697.11908937</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>722465907.39236546</c:v>
+                  <c:v>631294572.8514111</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>744465048.75484335</c:v>
+                  <c:v>637984108.1665597</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>663758995.57651436</c:v>
+                  <c:v>667541325.0782249</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>693746724.02089143</c:v>
+                  <c:v>757344004.95768011</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>769030353.48481762</c:v>
+                  <c:v>725685492.89085746</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -696,34 +696,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>334161607.2720179</c:v>
+                  <c:v>315804189.42996383</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>322855259.2979337</c:v>
+                  <c:v>307434632.62051517</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>356298274.69874299</c:v>
+                  <c:v>333184326.93666649</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>327751111.20573634</c:v>
+                  <c:v>359538479.32139218</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>329981990.07669067</c:v>
+                  <c:v>390285709.98276132</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>346494722.82543564</c:v>
+                  <c:v>402564103.74916875</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>398770675.51816463</c:v>
+                  <c:v>377405849.56199503</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>358591215.24249297</c:v>
+                  <c:v>340648666.21157545</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>401796597.58470345</c:v>
+                  <c:v>402285214.5380131</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>419328184.84190565</c:v>
+                  <c:v>417892522.16453439</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -770,34 +770,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>344035229.28476256</c:v>
+                  <c:v>449867903.82097661</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>391142458.22271389</c:v>
+                  <c:v>430976971.81612772</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>348604355.94792336</c:v>
+                  <c:v>421083322.20448852</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>393679101.61583698</c:v>
+                  <c:v>374007214.57592791</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>424450688.46772766</c:v>
+                  <c:v>400135903.70491248</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>412416119.8504374</c:v>
+                  <c:v>407466241.99841297</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>420945022.89417404</c:v>
+                  <c:v>408720007.50686431</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>450490847.44617671</c:v>
+                  <c:v>407827597.23438323</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>463726205.57963371</c:v>
+                  <c:v>349990551.18024623</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>435009464.81535572</c:v>
+                  <c:v>472720841.86251247</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -844,34 +844,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>286585048.41629392</c:v>
+                  <c:v>325602085.99996263</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>293608299.17772633</c:v>
+                  <c:v>317824203.00978869</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>317149045.99138379</c:v>
+                  <c:v>339636905.00294036</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>327014878.38268864</c:v>
+                  <c:v>337903547.41550303</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>336619627.86034638</c:v>
+                  <c:v>360246905.66393006</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>338667459.60914391</c:v>
+                  <c:v>366909200.58424103</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>383050933.28152722</c:v>
+                  <c:v>352892475.03423172</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>394077699.67294812</c:v>
+                  <c:v>398952421.15679967</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>435516907.66148931</c:v>
+                  <c:v>403596167.58389676</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>426722654.44961953</c:v>
+                  <c:v>387444452.78617281</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -918,34 +918,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>612594178.13352978</c:v>
+                  <c:v>716469135.2208643</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>578552808.84886742</c:v>
+                  <c:v>609821971.85227132</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>804434457.72079349</c:v>
+                  <c:v>695301475.81519341</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>622347907.45734739</c:v>
+                  <c:v>762464447.93890333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>797050394.14084923</c:v>
+                  <c:v>686389314.4452064</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>761047792.5542922</c:v>
+                  <c:v>799985931.68116021</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>845891380.52937686</c:v>
+                  <c:v>831863821.14259303</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>935343794.73410392</c:v>
+                  <c:v>873350186.74147618</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>864053553.89152241</c:v>
+                  <c:v>816658245.66131377</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>970430798.10298693</c:v>
+                  <c:v>962728529.51436865</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -992,34 +992,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>27360022.551898535</c:v>
+                  <c:v>31963266.345840931</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>35671995.023775443</c:v>
+                  <c:v>37221300.311860926</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40957965.06674134</c:v>
+                  <c:v>40900242.142210245</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46651821.38484703</c:v>
+                  <c:v>46648830.091460817</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>52037652.38280721</c:v>
+                  <c:v>51958960.220131822</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>58485474.245817833</c:v>
+                  <c:v>55169936.314006709</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67839325.216113374</c:v>
+                  <c:v>67707718.14164719</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>70647584.994573519</c:v>
+                  <c:v>72924338.547077373</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>83688572.811029285</c:v>
+                  <c:v>82191336.158397973</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>91343968.710075229</c:v>
+                  <c:v>90347937.70977132</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1066,34 +1066,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>205345673.76967528</c:v>
+                  <c:v>180626332.14641702</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>190512087.12484357</c:v>
+                  <c:v>234903455.59618309</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>267314617.84087193</c:v>
+                  <c:v>251984068.42984644</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>247533526.86054593</c:v>
+                  <c:v>239942103.58603629</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>328611798.83259988</c:v>
+                  <c:v>344365641.33358532</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>369108084.02593571</c:v>
+                  <c:v>377272561.38604409</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>438429986.68232673</c:v>
+                  <c:v>423357966.73157269</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>507323170.41951501</c:v>
+                  <c:v>567729050.62302148</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>594007843.33068144</c:v>
+                  <c:v>605786630.78349292</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>731926952.29417491</c:v>
+                  <c:v>791598901.25984669</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1140,34 +1140,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>224986828.00133488</c:v>
+                  <c:v>229617047.20396319</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>253236124.44606084</c:v>
+                  <c:v>240945752.67308432</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>252829865.25797909</c:v>
+                  <c:v>276233823.85737103</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>299137152.53839397</c:v>
+                  <c:v>314594025.93042862</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>339926643.43062532</c:v>
+                  <c:v>321897015.9009065</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>369443410.5810349</c:v>
+                  <c:v>386260327.82587272</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>402155465.65981758</c:v>
+                  <c:v>405501499.43285483</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>441686216.20688999</c:v>
+                  <c:v>458134082.10548717</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>484572073.16770411</c:v>
+                  <c:v>470477084.71559083</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>413676643.20716715</c:v>
+                  <c:v>428131633.6187433</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1978,10 +1978,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2838,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3015,10 +3011,85 @@
         <v>10522073.383424819</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>71923046.962598905</v>
+      </c>
+      <c r="B12">
+        <v>115096778.759151</v>
+      </c>
+      <c r="C12">
+        <f t="shared" ref="C12:C16" si="2">AVERAGE(A12:B12)</f>
+        <v>93509912.860874951</v>
+      </c>
+      <c r="D12" s="4">
+        <f>(B12-C12)/1.96</f>
+        <v>11013707.090957167</v>
+      </c>
+    </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
+      <c r="A13">
+        <v>76487378.491970494</v>
+      </c>
+      <c r="B13">
+        <v>123658050.519238</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="2"/>
+        <v>100072714.50560424</v>
+      </c>
+      <c r="D13" s="4">
+        <f t="shared" ref="D13:D16" si="3">(B13-C13)/1.96</f>
+        <v>12033334.70083355</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>81051710.021342203</v>
+      </c>
+      <c r="B14">
+        <v>132219322.27932701</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="2"/>
+        <v>106635516.1503346</v>
+      </c>
+      <c r="D14" s="4">
+        <f t="shared" si="3"/>
+        <v>13052962.310710413</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>85616041.550713807</v>
+      </c>
+      <c r="B15">
+        <v>140780594.03941399</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="2"/>
+        <v>113198317.7950639</v>
+      </c>
+      <c r="D15" s="4">
+        <f t="shared" si="3"/>
+        <v>14072589.920586782</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>90180373.080085397</v>
+      </c>
+      <c r="B16">
+        <v>149341865.79950199</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="2"/>
+        <v>119761119.43979369</v>
+      </c>
+      <c r="D16" s="4">
+        <f t="shared" si="3"/>
+        <v>15092217.530463416</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3075,43 +3146,43 @@
       </c>
       <c r="B2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C2,Measles!$D$2)</f>
-        <v>380279116.3628819</v>
+        <v>427844524.08335775</v>
       </c>
       <c r="C2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C3,Measles!$D$2)</f>
-        <v>448989663.26277512</v>
+        <v>266493540.45622987</v>
       </c>
       <c r="D2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C4,Measles!$D$2)</f>
-        <v>579693559.67794991</v>
+        <v>690921430.33690572</v>
       </c>
       <c r="E2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C5,Measles!$D$2)</f>
-        <v>477216801.40458322</v>
+        <v>608559229.60524082</v>
       </c>
       <c r="F2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C6,Measles!$D$2)</f>
-        <v>524049735.38377869</v>
+        <v>663849922.05193794</v>
       </c>
       <c r="G2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C7,Measles!$D$2)</f>
-        <v>786493791.26628435</v>
+        <v>720017052.81562459</v>
       </c>
       <c r="H2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C8,Measles!$D$2)</f>
-        <v>792703264.83761966</v>
+        <v>889418994.55034482</v>
       </c>
       <c r="I2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C9,Measles!$D$2)</f>
-        <v>837398630.38757217</v>
+        <v>904042059.50542402</v>
       </c>
       <c r="J2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C10,Measles!$D$2)</f>
-        <v>1002521692.9763725</v>
+        <v>1015447126.9340428</v>
       </c>
       <c r="K2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C11,Measles!$D$2)</f>
-        <v>1042180640.7550312</v>
+        <v>924995113.19309568</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
@@ -3120,43 +3191,43 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C2,Mumps!$D$2)</f>
-        <v>32802801.1819687</v>
+        <v>32215325.210729256</v>
       </c>
       <c r="C3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C3,Mumps!$D$2)</f>
-        <v>32297080.572214447</v>
+        <v>45516332.979260825</v>
       </c>
       <c r="D3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C4,Mumps!$D$2)</f>
-        <v>36664014.975054443</v>
+        <v>33898087.031309105</v>
       </c>
       <c r="E3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C5,Mumps!$D$2)</f>
-        <v>35606772.83373329</v>
+        <v>42814676.437276535</v>
       </c>
       <c r="F3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C6,Mumps!$D$2)</f>
-        <v>28353686.142964706</v>
+        <v>36449281.749024712</v>
       </c>
       <c r="G3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C7,Mumps!$D$2)</f>
-        <v>46353460.324733652</v>
+        <v>34376475.810845077</v>
       </c>
       <c r="H3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C8,Mumps!$D$2)</f>
-        <v>47386539.516075164</v>
+        <v>39757843.010042816</v>
       </c>
       <c r="I3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C9,Mumps!$D$2)</f>
-        <v>48049849.411365598</v>
+        <v>49608710.232102938</v>
       </c>
       <c r="J3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C10,Mumps!$D$2)</f>
-        <v>57006990.622826666</v>
+        <v>64076046.965096839</v>
       </c>
       <c r="K3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C11,Mumps!$D$2)</f>
-        <v>71338965.681571722</v>
+        <v>53151222.967799768</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -3165,43 +3236,43 @@
       </c>
       <c r="B4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C2,Rubella!$D$2)</f>
-        <v>455737876.75224012</v>
+        <v>321465048.4790833</v>
       </c>
       <c r="C4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C3,Rubella!$D$2)</f>
-        <v>279191668.70165825</v>
+        <v>338050229.20354372</v>
       </c>
       <c r="D4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C4,Rubella!$D$2)</f>
-        <v>491718464.82244426</v>
+        <v>383103937.96252614</v>
       </c>
       <c r="E4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C5,Rubella!$D$2)</f>
-        <v>321478288.58388901</v>
+        <v>566246441.65829504</v>
       </c>
       <c r="F4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C6,Rubella!$D$2)</f>
-        <v>582569187.24174964</v>
+        <v>462931671.903368</v>
       </c>
       <c r="G4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C7,Rubella!$D$2)</f>
-        <v>676324219.36442959</v>
+        <v>678288191.2504704</v>
       </c>
       <c r="H4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C8,Rubella!$D$2)</f>
-        <v>707046972.46634114</v>
+        <v>685059803.96362448</v>
       </c>
       <c r="I4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C9,Rubella!$D$2)</f>
-        <v>696541735.38053691</v>
+        <v>481911360.12481743</v>
       </c>
       <c r="J4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C10,Rubella!$D$2)</f>
-        <v>729825228.35502946</v>
+        <v>628165183.97071981</v>
       </c>
       <c r="K4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C11,Rubella!$D$2)</f>
-        <v>912144063.31862998</v>
+        <v>706453621.3172642</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -3210,43 +3281,43 @@
       </c>
       <c r="B5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C2,Diphtheria!$D$2)</f>
-        <v>730027462.43859041</v>
+        <v>625306808.80609596</v>
       </c>
       <c r="C5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C3,Diphtheria!$D$2)</f>
-        <v>748870069.02099586</v>
+        <v>574773030.64024889</v>
       </c>
       <c r="D5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C4,Diphtheria!$D$2)</f>
-        <v>857570894.05129778</v>
+        <v>723594153.53824306</v>
       </c>
       <c r="E5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C5,Diphtheria!$D$2)</f>
-        <v>841796851.68876898</v>
+        <v>840827455.21154118</v>
       </c>
       <c r="F5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C6,Diphtheria!$D$2)</f>
-        <v>940427660.20165586</v>
+        <v>839566408.24645913</v>
       </c>
       <c r="G5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C8,Diphtheria!$D$2)</f>
-        <v>997410651.78942442</v>
+        <v>1175682702.2142451</v>
       </c>
       <c r="H5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C9,Diphtheria!$D$2)</f>
-        <v>1342376979.3438168</v>
+        <v>1345041665.9302816</v>
       </c>
       <c r="I5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1609134848.1879845</v>
+        <v>1635771765.4634292</v>
       </c>
       <c r="J5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1583518014.6048779</v>
+        <v>1608781146.4265878</v>
       </c>
       <c r="K5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C11,Diphtheria!$D$2)</f>
-        <v>1863693054.9682305</v>
+        <v>1925303189.7746534</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
@@ -3255,43 +3326,43 @@
       </c>
       <c r="B6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C2,Tetanus!$D$2)</f>
-        <v>665645372.21190369</v>
+        <v>638898240.21864259</v>
       </c>
       <c r="C6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C3,Tetanus!$D$2)</f>
-        <v>635600563.96215916</v>
+        <v>645057838.57984638</v>
       </c>
       <c r="D6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C4,Tetanus!$D$2)</f>
-        <v>726256426.06573796</v>
+        <v>635282685.42925298</v>
       </c>
       <c r="E6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C5,Tetanus!$D$2)</f>
-        <v>709842146.89628315</v>
+        <v>699956110.31624317</v>
       </c>
       <c r="F6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C6,Tetanus!$D$2)</f>
-        <v>678579538.7353512</v>
+        <v>709104697.11908937</v>
       </c>
       <c r="G6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C7,Tetanus!$D$2)</f>
-        <v>722465907.39236546</v>
+        <v>631294572.8514111</v>
       </c>
       <c r="H6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C8,Tetanus!$D$2)</f>
-        <v>744465048.75484335</v>
+        <v>637984108.1665597</v>
       </c>
       <c r="I6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C9,Tetanus!$D$2)</f>
-        <v>663758995.57651436</v>
+        <v>667541325.0782249</v>
       </c>
       <c r="J6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C10,Tetanus!$D$2)</f>
-        <v>693746724.02089143</v>
+        <v>757344004.95768011</v>
       </c>
       <c r="K6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C11,Tetanus!$D$2)</f>
-        <v>769030353.48481762</v>
+        <v>725685492.89085746</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -3300,43 +3371,43 @@
       </c>
       <c r="B7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>334161607.2720179</v>
+        <v>315804189.42996383</v>
       </c>
       <c r="C7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>322855259.2979337</v>
+        <v>307434632.62051517</v>
       </c>
       <c r="D7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C4,Pertussis!$D$2)</f>
-        <v>356298274.69874299</v>
+        <v>333184326.93666649</v>
       </c>
       <c r="E7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C5,Pertussis!$D$2)</f>
-        <v>327751111.20573634</v>
+        <v>359538479.32139218</v>
       </c>
       <c r="F7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C6,Pertussis!$D$2)</f>
-        <v>329981990.07669067</v>
+        <v>390285709.98276132</v>
       </c>
       <c r="G7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C7,Pertussis!$D$2)</f>
-        <v>346494722.82543564</v>
+        <v>402564103.74916875</v>
       </c>
       <c r="H7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C8,Pertussis!$D$2)</f>
-        <v>398770675.51816463</v>
+        <v>377405849.56199503</v>
       </c>
       <c r="I7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C9,Pertussis!$D$2)</f>
-        <v>358591215.24249297</v>
+        <v>340648666.21157545</v>
       </c>
       <c r="J7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C10,Pertussis!$D$2)</f>
-        <v>401796597.58470345</v>
+        <v>402285214.5380131</v>
       </c>
       <c r="K7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C11,Pertussis!$D$2)</f>
-        <v>419328184.84190565</v>
+        <v>417892522.16453439</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
@@ -3345,43 +3416,43 @@
       </c>
       <c r="B8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C2,Hepatitis_B!$D$2)</f>
-        <v>344035229.28476256</v>
+        <v>457483356.99579835</v>
       </c>
       <c r="C8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C3,Hepatitis_B!$D$2)</f>
-        <v>391142458.22271389</v>
+        <v>430976971.81612772</v>
       </c>
       <c r="D8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C4,Hepatitis_B!$D$2)</f>
-        <v>348604355.94792336</v>
+        <v>421083322.20448852</v>
       </c>
       <c r="E8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C5,Hepatitis_B!$D$2)</f>
-        <v>393679101.61583698</v>
+        <v>374007214.57592791</v>
       </c>
       <c r="F8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C6,Hepatitis_B!$D$2)</f>
-        <v>424450688.46772766</v>
+        <v>400135903.70491248</v>
       </c>
       <c r="G8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C7,Hepatitis_B!$D$2)</f>
-        <v>412416119.8504374</v>
+        <v>407466241.99841297</v>
       </c>
       <c r="H8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C8,Hepatitis_B!$D$2)</f>
-        <v>420945022.89417404</v>
+        <v>408720007.50686431</v>
       </c>
       <c r="I8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C9,Hepatitis_B!$D$2)</f>
-        <v>450490847.44617671</v>
+        <v>407827597.23438323</v>
       </c>
       <c r="J8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C10,Hepatitis_B!$D$2)</f>
-        <v>463726205.57963371</v>
+        <v>349990551.18024623</v>
       </c>
       <c r="K8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,Hepatitis_B!$D$2)</f>
-        <v>435009464.81535572</v>
+        <v>472720841.86251247</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
@@ -3390,43 +3461,43 @@
       </c>
       <c r="B9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C2,Hib!$D$2)</f>
-        <v>286585048.41629392</v>
+        <v>325602085.99996263</v>
       </c>
       <c r="C9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C3,Hib!$D$2)</f>
-        <v>293608299.17772633</v>
+        <v>317824203.00978869</v>
       </c>
       <c r="D9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C4,Hib!$D$2)</f>
-        <v>317149045.99138379</v>
+        <v>339636905.00294036</v>
       </c>
       <c r="E9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C5,Hib!$D$2)</f>
-        <v>327014878.38268864</v>
+        <v>337903547.41550303</v>
       </c>
       <c r="F9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C6,Hib!$D$2)</f>
-        <v>336619627.86034638</v>
+        <v>360246905.66393006</v>
       </c>
       <c r="G9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C7,Hib!$D$2)</f>
-        <v>338667459.60914391</v>
+        <v>366909200.58424103</v>
       </c>
       <c r="H9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C8,Hib!$D$2)</f>
-        <v>383050933.28152722</v>
+        <v>352892475.03423172</v>
       </c>
       <c r="I9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C9,Hib!$D$2)</f>
-        <v>394077699.67294812</v>
+        <v>398952421.15679967</v>
       </c>
       <c r="J9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C10,Hib!$D$2)</f>
-        <v>435516907.66148931</v>
+        <v>403596167.58389676</v>
       </c>
       <c r="K9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C11,Hib!$D$2)</f>
-        <v>426722654.44961953</v>
+        <v>387444452.78617281</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
@@ -3435,43 +3506,43 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C2,Polio!$D$2)</f>
-        <v>612594178.13352978</v>
+        <v>736527737.92395699</v>
       </c>
       <c r="C10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C3,Polio!$D$2)</f>
-        <v>578552808.84886742</v>
+        <v>609821971.85227132</v>
       </c>
       <c r="D10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C4,Polio!$D$2)</f>
-        <v>804434457.72079349</v>
+        <v>695301475.81519341</v>
       </c>
       <c r="E10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C5,Polio!$D$2)</f>
-        <v>622347907.45734739</v>
+        <v>762464447.93890333</v>
       </c>
       <c r="F10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C6,Polio!$D$2)</f>
-        <v>797050394.14084923</v>
+        <v>686389314.4452064</v>
       </c>
       <c r="G10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C7,Polio!$D$2)</f>
-        <v>761047792.5542922</v>
+        <v>799985931.68116021</v>
       </c>
       <c r="H10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C8,Polio!$D$2)</f>
-        <v>845891380.52937686</v>
+        <v>831863821.14259303</v>
       </c>
       <c r="I10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C9,Polio!$D$2)</f>
-        <v>935343794.73410392</v>
+        <v>873350186.74147618</v>
       </c>
       <c r="J10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C10,Polio!$D$2)</f>
-        <v>864053553.89152241</v>
+        <v>816658245.66131377</v>
       </c>
       <c r="K10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C11,Polio!$D$2)</f>
-        <v>970430798.10298693</v>
+        <v>962728529.51436865</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
@@ -3480,43 +3551,43 @@
       </c>
       <c r="B11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C2,HPV!$D$2)</f>
-        <v>27360022.551898535</v>
+        <v>32323300.612997241</v>
       </c>
       <c r="C11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C3,HPV!$D$2)</f>
-        <v>35671995.023775443</v>
+        <v>37221300.311860926</v>
       </c>
       <c r="D11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C4,HPV!$D$2)</f>
-        <v>40957965.06674134</v>
+        <v>40900242.142210245</v>
       </c>
       <c r="E11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C5,HPV!$D$2)</f>
-        <v>46651821.38484703</v>
+        <v>46648830.091460817</v>
       </c>
       <c r="F11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C6,HPV!$D$2)</f>
-        <v>52037652.38280721</v>
+        <v>51958960.220131822</v>
       </c>
       <c r="G11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C7,HPV!$D$2)</f>
-        <v>58485474.245817833</v>
+        <v>55169936.314006709</v>
       </c>
       <c r="H11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C8,HPV!$D$2)</f>
-        <v>67839325.216113374</v>
+        <v>67707718.14164719</v>
       </c>
       <c r="I11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C9,HPV!$D$2)</f>
-        <v>70647584.994573519</v>
+        <v>72924338.547077373</v>
       </c>
       <c r="J11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C10,HPV!$D$2)</f>
-        <v>83688572.811029285</v>
+        <v>82191336.158397973</v>
       </c>
       <c r="K11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C11,HPV!$D$2)</f>
-        <v>91343968.710075229</v>
+        <v>90347937.70977132</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
@@ -3525,43 +3596,43 @@
       </c>
       <c r="B12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C2,Rotavirus!$D$2)</f>
-        <v>205345673.76967528</v>
+        <v>180626332.14641702</v>
       </c>
       <c r="C12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C3,Rotavirus!$D$2)</f>
-        <v>190512087.12484357</v>
+        <v>234903455.59618309</v>
       </c>
       <c r="D12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C4,Rotavirus!$D$2)</f>
-        <v>267314617.84087193</v>
+        <v>251984068.42984644</v>
       </c>
       <c r="E12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C5,Rotavirus!$D$2)</f>
-        <v>247533526.86054593</v>
+        <v>239942103.58603629</v>
       </c>
       <c r="F12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C6,Rotavirus!$D$2)</f>
-        <v>328611798.83259988</v>
+        <v>344365641.33358532</v>
       </c>
       <c r="G12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C7,Rotavirus!$D$2)</f>
-        <v>369108084.02593571</v>
+        <v>377272561.38604409</v>
       </c>
       <c r="H12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C8,Rotavirus!$D$2)</f>
-        <v>438429986.68232673</v>
+        <v>423357966.73157269</v>
       </c>
       <c r="I12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C9,Rotavirus!$D$2)</f>
-        <v>507323170.41951501</v>
+        <v>567729050.62302148</v>
       </c>
       <c r="J12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C10,Rotavirus!$D$2)</f>
-        <v>594007843.33068144</v>
+        <v>605786630.78349292</v>
       </c>
       <c r="K12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C11,Rotavirus!$D$2)</f>
-        <v>731926952.29417491</v>
+        <v>791598901.25984669</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
@@ -3570,43 +3641,43 @@
       </c>
       <c r="B13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C2,PCV!$D$2)</f>
-        <v>224986828.00133488</v>
+        <v>229617047.20396319</v>
       </c>
       <c r="C13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C3,PCV!$D$2)</f>
-        <v>253236124.44606084</v>
+        <v>240945752.67308432</v>
       </c>
       <c r="D13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C4,PCV!$D$2)</f>
-        <v>252829865.25797909</v>
+        <v>276233823.85737103</v>
       </c>
       <c r="E13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C5,PCV!$D$2)</f>
-        <v>299137152.53839397</v>
+        <v>314594025.93042862</v>
       </c>
       <c r="F13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C6,PCV!$D$2)</f>
-        <v>339926643.43062532</v>
+        <v>321897015.9009065</v>
       </c>
       <c r="G13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C7,PCV!$D$2)</f>
-        <v>369443410.5810349</v>
+        <v>386260327.82587272</v>
       </c>
       <c r="H13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C8,PCV!$D$2)</f>
-        <v>402155465.65981758</v>
+        <v>405501499.43285483</v>
       </c>
       <c r="I13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C9,PCV!$D$2)</f>
-        <v>441686216.20688999</v>
+        <v>458134082.10548717</v>
       </c>
       <c r="J13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C10,PCV!$D$2)</f>
-        <v>484572073.16770411</v>
+        <v>470477084.71559083</v>
       </c>
       <c r="K13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,PCV!$D$2)</f>
-        <v>413676643.20716715</v>
+        <v>428131633.6187433</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
@@ -3615,43 +3686,43 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(B2&gt;Measles!B2,Measles!B2,IF(Scenario_data!B2 &lt;Measles!A2,Measles!A2,Scenario_data!B2))</f>
-        <v>380279116.3628819</v>
+        <v>427844524.08335775</v>
       </c>
       <c r="C15" s="7">
         <f ca="1">IF(C2&gt;Measles!B3,Measles!B3,IF(Scenario_data!C2 &lt;Measles!A3,Measles!A3,Scenario_data!C2))</f>
-        <v>448989663.26277512</v>
+        <v>266493540.45622987</v>
       </c>
       <c r="D15" s="7">
         <f ca="1">IF(D2&gt;Measles!B4,Measles!B4,IF(Scenario_data!D2 &lt;Measles!A4,Measles!A4,Scenario_data!D2))</f>
-        <v>579693559.67794991</v>
+        <v>690921430.33690572</v>
       </c>
       <c r="E15" s="7">
         <f ca="1">IF(E2&gt;Measles!B5,Measles!B5,IF(Scenario_data!E2 &lt;Measles!A5,Measles!A5,Scenario_data!E2))</f>
-        <v>477216801.40458322</v>
+        <v>608559229.60524082</v>
       </c>
       <c r="F15" s="7">
         <f ca="1">IF(F2&gt;Measles!B6,Measles!B6,IF(Scenario_data!F2 &lt;Measles!A6,Measles!A6,Scenario_data!F2))</f>
-        <v>524049735.38377869</v>
+        <v>663849922.05193794</v>
       </c>
       <c r="G15" s="7">
         <f ca="1">IF(G2&gt;Measles!B7,Measles!B7,IF(Scenario_data!G2 &lt;Measles!A7,Measles!A7,Scenario_data!G2))</f>
-        <v>786493791.26628435</v>
+        <v>720017052.81562459</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">IF(H2&gt;Measles!B8,Measles!B8,IF(Scenario_data!H2 &lt;Measles!A8,Measles!A8,Scenario_data!H2))</f>
-        <v>792703264.83761966</v>
+        <v>889418994.55034482</v>
       </c>
       <c r="I15" s="7">
         <f ca="1">IF(I2&gt;Measles!B9,Measles!B9,IF(Scenario_data!I2 &lt;Measles!A9,Measles!A9,Scenario_data!I2))</f>
-        <v>837398630.38757217</v>
+        <v>904042059.50542402</v>
       </c>
       <c r="J15" s="7">
         <f ca="1">IF(J2&gt;Measles!B10,Measles!B10,IF(Scenario_data!J2 &lt;Measles!A10,Measles!A10,Scenario_data!J2))</f>
-        <v>1002521692.9763725</v>
+        <v>1015447126.9340428</v>
       </c>
       <c r="K15" s="7">
         <f ca="1">IF(K2&gt;Measles!B11,Measles!B11,IF(Scenario_data!K2 &lt;Measles!A11,Measles!A11,Scenario_data!K2))</f>
-        <v>1042180640.7550312</v>
+        <v>924995113.19309568</v>
       </c>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
@@ -3662,43 +3733,43 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(B3&gt;Mumps!B2,Mumps!B2,IF(Scenario_data!B3 &lt;Mumps!A2,Mumps!A2,Scenario_data!B3))</f>
-        <v>32802801.1819687</v>
+        <v>32215325.210729256</v>
       </c>
       <c r="C16" s="7">
         <f ca="1">IF(C3&gt;Mumps!B3,Mumps!B3,IF(Scenario_data!C3 &lt;Mumps!A3,Mumps!A3,Scenario_data!C3))</f>
-        <v>32297080.572214447</v>
+        <v>45516332.979260825</v>
       </c>
       <c r="D16" s="7">
         <f ca="1">IF(D3&gt;Mumps!B4,Mumps!B4,IF(Scenario_data!D3 &lt;Mumps!A4,Mumps!A4,Scenario_data!D3))</f>
-        <v>36664014.975054443</v>
+        <v>33898087.031309105</v>
       </c>
       <c r="E16" s="7">
         <f ca="1">IF(E3&gt;Mumps!B5,Mumps!B5,IF(Scenario_data!E3 &lt;Mumps!A5,Mumps!A5,Scenario_data!E3))</f>
-        <v>35606772.83373329</v>
+        <v>42814676.437276535</v>
       </c>
       <c r="F16" s="7">
         <f ca="1">IF(F3&gt;Mumps!B6,Mumps!B6,IF(Scenario_data!F3 &lt;Mumps!A6,Mumps!A6,Scenario_data!F3))</f>
-        <v>28353686.142964706</v>
+        <v>36449281.749024712</v>
       </c>
       <c r="G16" s="7">
         <f ca="1">IF(G3&gt;Mumps!B7,Mumps!B7,IF(Scenario_data!G3 &lt;Mumps!A7,Mumps!A7,Scenario_data!G3))</f>
-        <v>46353460.324733652</v>
+        <v>34376475.810845077</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">IF(H3&gt;Mumps!B8,Mumps!B8,IF(Scenario_data!H3 &lt;Mumps!A8,Mumps!A8,Scenario_data!H3))</f>
-        <v>47386539.516075164</v>
+        <v>39757843.010042816</v>
       </c>
       <c r="I16" s="7">
         <f ca="1">IF(I3&gt;Mumps!B9,Mumps!B9,IF(Scenario_data!I3 &lt;Mumps!A9,Mumps!A9,Scenario_data!I3))</f>
-        <v>48049849.411365598</v>
+        <v>49608710.232102938</v>
       </c>
       <c r="J16" s="7">
         <f ca="1">IF(J3&gt;Mumps!B10,Mumps!B10,IF(Scenario_data!J3 &lt;Mumps!A10,Mumps!A10,Scenario_data!J3))</f>
-        <v>57006990.622826666</v>
+        <v>64076046.965096839</v>
       </c>
       <c r="K16" s="7">
         <f ca="1">IF(K3&gt;Mumps!B11,Mumps!B11,IF(Scenario_data!K3 &lt;Mumps!A11,Mumps!A11,Scenario_data!K3))</f>
-        <v>71338965.681571722</v>
+        <v>53151222.967799768</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -3707,43 +3778,43 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(B4&gt;Rubella!B2,Rubella!B2,IF(Scenario_data!B4 &lt;Rubella!A2,Rubella!A2,Scenario_data!B4))</f>
-        <v>455737876.75224012</v>
+        <v>321465048.4790833</v>
       </c>
       <c r="C17" s="7">
         <f ca="1">IF(C4&gt;Rubella!B3,Rubella!B3,IF(Scenario_data!C4 &lt;Rubella!A3,Rubella!A3,Scenario_data!C4))</f>
-        <v>279191668.70165825</v>
+        <v>338050229.20354372</v>
       </c>
       <c r="D17" s="7">
         <f ca="1">IF(D4&gt;Rubella!B4,Rubella!B4,IF(Scenario_data!D4 &lt;Rubella!A4,Rubella!A4,Scenario_data!D4))</f>
-        <v>491718464.82244426</v>
+        <v>383103937.96252614</v>
       </c>
       <c r="E17" s="7">
         <f ca="1">IF(E4&gt;Rubella!B5,Rubella!B5,IF(Scenario_data!E4 &lt;Rubella!A5,Rubella!A5,Scenario_data!E4))</f>
-        <v>321478288.58388901</v>
+        <v>566246441.65829504</v>
       </c>
       <c r="F17" s="7">
         <f ca="1">IF(F4&gt;Rubella!B6,Rubella!B6,IF(Scenario_data!F4 &lt;Rubella!A6,Rubella!A6,Scenario_data!F4))</f>
-        <v>582569187.24174964</v>
+        <v>462931671.903368</v>
       </c>
       <c r="G17" s="7">
         <f ca="1">IF(G4&gt;Rubella!B7,Rubella!B7,IF(Scenario_data!G4 &lt;Rubella!A7,Rubella!A7,Scenario_data!G4))</f>
-        <v>676324219.36442959</v>
+        <v>678288191.2504704</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">IF(H4&gt;Rubella!B8,Rubella!B8,IF(Scenario_data!H4 &lt;Rubella!A8,Rubella!A8,Scenario_data!H4))</f>
-        <v>707046972.46634114</v>
+        <v>685059803.96362448</v>
       </c>
       <c r="I17" s="7">
         <f ca="1">IF(I4&gt;Rubella!B9,Rubella!B9,IF(Scenario_data!I4 &lt;Rubella!A9,Rubella!A9,Scenario_data!I4))</f>
-        <v>696541735.38053691</v>
+        <v>481911360.12481743</v>
       </c>
       <c r="J17" s="7">
         <f ca="1">IF(J4&gt;Rubella!B10,Rubella!B10,IF(Scenario_data!J4 &lt;Rubella!A10,Rubella!A10,Scenario_data!J4))</f>
-        <v>729825228.35502946</v>
+        <v>628165183.97071981</v>
       </c>
       <c r="K17" s="7">
         <f ca="1">IF(K4&gt;Rubella!B12=1,Rubella!B11,IF(Scenario_data!K4 &lt;Rubella!A11,Rubella!A11,Scenario_data!K4))</f>
-        <v>912144063.31862998</v>
+        <v>706453621.3172642</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -3752,43 +3823,43 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(B5&gt;Diphtheria!B2,Diphtheria!B2,IF(Scenario_data!B5 &lt;Diphtheria!A2,Diphtheria!A2,Scenario_data!B5))</f>
-        <v>730027462.43859041</v>
+        <v>625306808.80609596</v>
       </c>
       <c r="C18" s="7">
         <f ca="1">IF(C5&gt;Diphtheria!B3,Diphtheria!B3,IF(Scenario_data!C5 &lt;Diphtheria!A3,Diphtheria!A3,Scenario_data!C5))</f>
-        <v>748870069.02099586</v>
+        <v>574773030.64024889</v>
       </c>
       <c r="D18" s="7">
         <f ca="1">IF(D5&gt;Diphtheria!B4,Diphtheria!B4,IF(Scenario_data!D5 &lt;Diphtheria!A4,Diphtheria!A4,Scenario_data!D5))</f>
-        <v>857570894.05129778</v>
+        <v>723594153.53824306</v>
       </c>
       <c r="E18" s="7">
         <f ca="1">IF(E5&gt;Diphtheria!B5,Diphtheria!B5,IF(Scenario_data!E5 &lt;Diphtheria!A5,Diphtheria!A5,Scenario_data!E5))</f>
-        <v>841796851.68876898</v>
+        <v>840827455.21154118</v>
       </c>
       <c r="F18" s="7">
         <f ca="1">IF(F5&gt;Diphtheria!B6,Diphtheria!B6,IF(Scenario_data!F5 &lt;Diphtheria!A6,Diphtheria!A6,Scenario_data!F5))</f>
-        <v>940427660.20165586</v>
+        <v>839566408.24645913</v>
       </c>
       <c r="G18" s="7">
         <f ca="1">IF(G5&gt;Diphtheria!B7,Diphtheria!B7,IF(Scenario_data!G5 &lt;Diphtheria!A7,Diphtheria!A7,Scenario_data!G5))</f>
-        <v>997410651.78942442</v>
+        <v>1175682702.2142451</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">IF(H5&gt;Diphtheria!B8,Diphtheria!B8,IF(Scenario_data!H5 &lt;Diphtheria!A8,Diphtheria!A8,Scenario_data!H5))</f>
-        <v>1342376979.3438168</v>
+        <v>1345041665.9302816</v>
       </c>
       <c r="I18" s="7">
         <f ca="1">IF(I5&gt;Diphtheria!B9,Diphtheria!B9,IF(Scenario_data!I5 &lt;Diphtheria!A9,Diphtheria!A9,Scenario_data!I5))</f>
-        <v>1609134848.1879845</v>
+        <v>1635771765.4634292</v>
       </c>
       <c r="J18" s="7">
         <f ca="1">IF(J5&gt;Diphtheria!B10,Diphtheria!B10,IF(Scenario_data!J5 &lt;Diphtheria!A10,Diphtheria!A10,Scenario_data!J5))</f>
-        <v>1583518014.6048779</v>
+        <v>1608781146.4265878</v>
       </c>
       <c r="K18" s="7">
         <f ca="1">IF(K5&gt;Diphtheria!B11,Diphtheria!B11,IF(Scenario_data!K5 &lt;Diphtheria!A11,Diphtheria!A11,Scenario_data!K5))</f>
-        <v>1863693054.9682305</v>
+        <v>1925303189.7746534</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -3797,43 +3868,43 @@
       </c>
       <c r="B19" s="7">
         <f ca="1">IF(B6&gt;Tetanus!B2,Tetanus!B2,IF(Scenario_data!B6 &lt;Tetanus!A2,Tetanus!A2,Scenario_data!B6))</f>
-        <v>665645372.21190369</v>
+        <v>638898240.21864259</v>
       </c>
       <c r="C19" s="7">
         <f ca="1">IF(C6&gt;Tetanus!B3,Tetanus!B3,IF(Scenario_data!C6 &lt;Tetanus!A3,Tetanus!A3,Scenario_data!C6))</f>
-        <v>635600563.96215916</v>
+        <v>645057838.57984638</v>
       </c>
       <c r="D19" s="7">
         <f ca="1">IF(D6&gt;Tetanus!B4,Tetanus!B4,IF(Scenario_data!D6 &lt;Tetanus!A4,Tetanus!A4,Scenario_data!D6))</f>
-        <v>726256426.06573796</v>
+        <v>635282685.42925298</v>
       </c>
       <c r="E19" s="7">
         <f ca="1">IF(E6&gt;Tetanus!B5,Tetanus!B5,IF(Scenario_data!E6 &lt;Tetanus!A5,Tetanus!A5,Scenario_data!E6))</f>
-        <v>709842146.89628315</v>
+        <v>699956110.31624317</v>
       </c>
       <c r="F19" s="7">
         <f ca="1">IF(F6&gt;Tetanus!B6,Tetanus!B6,IF(Scenario_data!F6 &lt;Tetanus!A6,Tetanus!A6,Scenario_data!F6))</f>
-        <v>678579538.7353512</v>
+        <v>709104697.11908937</v>
       </c>
       <c r="G19" s="7">
         <f ca="1">IF(G6&gt;Tetanus!B7,Tetanus!B7,IF(Scenario_data!G6 &lt;Tetanus!A7,Tetanus!A7,Scenario_data!G6))</f>
-        <v>722465907.39236546</v>
+        <v>631294572.8514111</v>
       </c>
       <c r="H19" s="7">
         <f ca="1">IF(H6&gt;Tetanus!B8,Tetanus!B8,IF(Scenario_data!H6 &lt;Tetanus!A8,Tetanus!A8,Scenario_data!H6))</f>
-        <v>744465048.75484335</v>
+        <v>637984108.1665597</v>
       </c>
       <c r="I19" s="7">
         <f ca="1">IF(I6&gt;Tetanus!B9,Tetanus!B9,IF(Scenario_data!I6 &lt;Tetanus!A9,Tetanus!A9,Scenario_data!I6))</f>
-        <v>663758995.57651436</v>
+        <v>667541325.0782249</v>
       </c>
       <c r="J19" s="7">
         <f ca="1">IF(J6&gt;Tetanus!B10,Tetanus!B10,IF(Scenario_data!J6 &lt;Tetanus!A10,Tetanus!A10,Scenario_data!J6))</f>
-        <v>693746724.02089143</v>
+        <v>757344004.95768011</v>
       </c>
       <c r="K19" s="7">
         <f ca="1">IF(K6&gt;Tetanus!B11,Tetanus!B11,IF(Scenario_data!K6 &lt;Tetanus!A11,Tetanus!A11,Scenario_data!K6))</f>
-        <v>769030353.48481762</v>
+        <v>725685492.89085746</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -3842,43 +3913,43 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IF(B7&gt;Pertussis!B2,Pertussis!B2,IF(Scenario_data!B7 &lt;Pertussis!A2,Pertussis!A2,Scenario_data!B7))</f>
-        <v>334161607.2720179</v>
+        <v>315804189.42996383</v>
       </c>
       <c r="C20" s="7">
         <f ca="1">IF(C7&gt;Pertussis!B3,Pertussis!B3,IF(Scenario_data!C7 &lt;Pertussis!A3,Pertussis!A3,Scenario_data!C7))</f>
-        <v>322855259.2979337</v>
+        <v>307434632.62051517</v>
       </c>
       <c r="D20" s="7">
         <f ca="1">IF(D7&gt;Pertussis!B4,Pertussis!B4,IF(Scenario_data!D7 &lt;Pertussis!A4,Pertussis!A4,Scenario_data!D7))</f>
-        <v>356298274.69874299</v>
+        <v>333184326.93666649</v>
       </c>
       <c r="E20" s="7">
         <f ca="1">IF(E7&gt;Pertussis!B5,Pertussis!B5,IF(Scenario_data!E7 &lt;Pertussis!A5,Pertussis!A5,Scenario_data!E7))</f>
-        <v>327751111.20573634</v>
+        <v>359538479.32139218</v>
       </c>
       <c r="F20" s="7">
         <f ca="1">IF(F7&gt;Pertussis!B6,Pertussis!B6,IF(Scenario_data!F7 &lt;Pertussis!A6,Pertussis!A6,Scenario_data!F7))</f>
-        <v>329981990.07669067</v>
+        <v>390285709.98276132</v>
       </c>
       <c r="G20" s="7">
         <f ca="1">IF(G7&gt;Pertussis!B7,Pertussis!B7,IF(Scenario_data!G7 &lt;Pertussis!A7,Pertussis!A7,Scenario_data!G7))</f>
-        <v>346494722.82543564</v>
+        <v>402564103.74916875</v>
       </c>
       <c r="H20" s="7">
         <f ca="1">IF(H7&gt;Pertussis!B8,Pertussis!B8,IF(Scenario_data!H7 &lt;Pertussis!A8,Pertussis!A8,Scenario_data!H7))</f>
-        <v>398770675.51816463</v>
+        <v>377405849.56199503</v>
       </c>
       <c r="I20" s="7">
         <f ca="1">IF(I7&gt;Pertussis!B9,Pertussis!B9,IF(Scenario_data!I7 &lt;Pertussis!A9,Pertussis!A9,Scenario_data!I7))</f>
-        <v>358591215.24249297</v>
+        <v>340648666.21157545</v>
       </c>
       <c r="J20" s="7">
         <f ca="1">IF(J7&gt;Pertussis!B10,Pertussis!B10,IF(Scenario_data!J7 &lt;Pertussis!A10,Pertussis!A10,Scenario_data!J7))</f>
-        <v>401796597.58470345</v>
+        <v>402285214.5380131</v>
       </c>
       <c r="K20" s="7">
         <f ca="1">IF(K7&gt;Pertussis!B11,Pertussis!B11,IF(Scenario_data!K7 &lt;Pertussis!A11,Pertussis!A11,Scenario_data!K7))</f>
-        <v>419328184.84190565</v>
+        <v>417892522.16453439</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -3887,43 +3958,43 @@
       </c>
       <c r="B21" s="7">
         <f ca="1">IF(B8&gt;Hepatitis_B!B2,Hepatitis_B!B2,IF(Scenario_data!B8 &lt;Hepatitis_B!A2,Hepatitis_B!A2,Scenario_data!B8))</f>
-        <v>344035229.28476256</v>
+        <v>449867903.82097661</v>
       </c>
       <c r="C21" s="7">
         <f ca="1">IF(C8&gt;Hepatitis_B!B3,Hepatitis_B!B3,IF(Scenario_data!C8 &lt;Hepatitis_B!A3,Hepatitis_B!A3,Scenario_data!C8))</f>
-        <v>391142458.22271389</v>
+        <v>430976971.81612772</v>
       </c>
       <c r="D21" s="7">
         <f ca="1">IF(D8&gt;Hepatitis_B!B4,Hepatitis_B!B4,IF(Scenario_data!D8 &lt;Hepatitis_B!A4,Hepatitis_B!A4,Scenario_data!D8))</f>
-        <v>348604355.94792336</v>
+        <v>421083322.20448852</v>
       </c>
       <c r="E21" s="7">
         <f ca="1">IF(E8&gt;Hepatitis_B!B5,Hepatitis_B!B5,IF(Scenario_data!E8 &lt;Hepatitis_B!A5,Hepatitis_B!A5,Scenario_data!E8))</f>
-        <v>393679101.61583698</v>
+        <v>374007214.57592791</v>
       </c>
       <c r="F21" s="7">
         <f ca="1">IF(F8&gt;Hepatitis_B!B6,Hepatitis_B!B6,IF(Scenario_data!F8 &lt;Hepatitis_B!A6,Hepatitis_B!A6,Scenario_data!F8))</f>
-        <v>424450688.46772766</v>
+        <v>400135903.70491248</v>
       </c>
       <c r="G21" s="7">
         <f ca="1">IF(G8&gt;Hepatitis_B!B7,Hepatitis_B!B7,IF(Scenario_data!G8 &lt;Hepatitis_B!A7,Hepatitis_B!A7,Scenario_data!G8))</f>
-        <v>412416119.8504374</v>
+        <v>407466241.99841297</v>
       </c>
       <c r="H21" s="7">
         <f ca="1">IF(H8&gt;Hepatitis_B!B8,Hepatitis_B!B8,IF(Scenario_data!H8 &lt;Hepatitis_B!A8,Hepatitis_B!A8,Scenario_data!H8))</f>
-        <v>420945022.89417404</v>
+        <v>408720007.50686431</v>
       </c>
       <c r="I21" s="7">
         <f ca="1">IF(I8&gt;Hepatitis_B!B9,Hepatitis_B!B9,IF(Scenario_data!I8 &lt;Hepatitis_B!A9,Hepatitis_B!A9,Scenario_data!I8))</f>
-        <v>450490847.44617671</v>
+        <v>407827597.23438323</v>
       </c>
       <c r="J21" s="7">
         <f ca="1">IF(J8&gt;Hepatitis_B!B10,Hepatitis_B!B10,IF(Scenario_data!J8 &lt;Hepatitis_B!A10,Hepatitis_B!A10,Scenario_data!J8))</f>
-        <v>463726205.57963371</v>
+        <v>349990551.18024623</v>
       </c>
       <c r="K21" s="7">
         <f ca="1">IF(K8&gt;Hepatitis_B!B11,Hepatitis_B!B11,IF(Scenario_data!K8 &lt;Hepatitis_B!A11,Hepatitis_B!A11,Scenario_data!K8))</f>
-        <v>435009464.81535572</v>
+        <v>472720841.86251247</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -3932,43 +4003,43 @@
       </c>
       <c r="B22" s="7">
         <f ca="1">IF(B9&gt;Hib!B2,Hib!B2,IF(Scenario_data!B9 &lt;Hib!A2,Hib!A2,Scenario_data!B9))</f>
-        <v>286585048.41629392</v>
+        <v>325602085.99996263</v>
       </c>
       <c r="C22" s="7">
         <f ca="1">IF(C9&gt;Hib!B3,Hib!B3,IF(Scenario_data!C9 &lt;Hib!A3,Hib!A3,Scenario_data!C9))</f>
-        <v>293608299.17772633</v>
+        <v>317824203.00978869</v>
       </c>
       <c r="D22" s="7">
         <f ca="1">IF(D9&gt;Hib!B4,Hib!B4,IF(Scenario_data!D9 &lt;Hib!A4,Hib!A4,Scenario_data!D9))</f>
-        <v>317149045.99138379</v>
+        <v>339636905.00294036</v>
       </c>
       <c r="E22" s="7">
         <f ca="1">IF(E9&gt;Hib!B5,Hib!B5,IF(Scenario_data!E9 &lt;Hib!A5,Hib!A5,Scenario_data!E9))</f>
-        <v>327014878.38268864</v>
+        <v>337903547.41550303</v>
       </c>
       <c r="F22" s="7">
         <f ca="1">IF(F9&gt;Hib!B6,Hib!B6,IF(Scenario_data!F9 &lt;Hib!A6,Hib!A6,Scenario_data!F9))</f>
-        <v>336619627.86034638</v>
+        <v>360246905.66393006</v>
       </c>
       <c r="G22" s="7">
         <f ca="1">IF(G9&gt;Hib!B7,Hib!B7,IF(Scenario_data!G9 &lt;Hib!A7,Hib!A7,Scenario_data!G9))</f>
-        <v>338667459.60914391</v>
+        <v>366909200.58424103</v>
       </c>
       <c r="H22" s="7">
         <f ca="1">IF(H9&gt;Hib!B8,Hib!B8,IF(Scenario_data!H9 &lt;Hib!A8,Hib!A8,Scenario_data!H9))</f>
-        <v>383050933.28152722</v>
+        <v>352892475.03423172</v>
       </c>
       <c r="I22" s="7">
         <f ca="1">IF(I9&gt;Hib!B9,Hib!B9,IF(Scenario_data!I9 &lt;Hib!A9,Hib!A9,Scenario_data!I9))</f>
-        <v>394077699.67294812</v>
+        <v>398952421.15679967</v>
       </c>
       <c r="J22" s="7">
         <f ca="1">IF(J9&gt;Hib!B10,Hib!B10,IF(Scenario_data!J9 &lt;Hib!A10,Hib!A10,Scenario_data!J9))</f>
-        <v>435516907.66148931</v>
+        <v>403596167.58389676</v>
       </c>
       <c r="K22" s="7">
         <f ca="1">IF(K9&gt;Hib!B11,Hib!B11,IF(Scenario_data!K9 &lt;Hib!A11,Hib!A11,Scenario_data!K9))</f>
-        <v>426722654.44961953</v>
+        <v>387444452.78617281</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -3977,43 +4048,43 @@
       </c>
       <c r="B23" s="7">
         <f ca="1">IF(B10&gt;Polio!B2,Polio!B2,IF(Scenario_data!B10 &lt;Polio!A2,Polio!A2,Scenario_data!B10))</f>
-        <v>612594178.13352978</v>
+        <v>716469135.2208643</v>
       </c>
       <c r="C23" s="7">
         <f ca="1">IF(C10&gt;Polio!B3,Polio!B3,IF(Scenario_data!C10 &lt;Polio!A3,Polio!A3,Scenario_data!C10))</f>
-        <v>578552808.84886742</v>
+        <v>609821971.85227132</v>
       </c>
       <c r="D23" s="7">
         <f ca="1">IF(D10&gt;Polio!B4,Polio!B4,IF(Scenario_data!D10 &lt;Polio!A4,Polio!A4,Scenario_data!D10))</f>
-        <v>804434457.72079349</v>
+        <v>695301475.81519341</v>
       </c>
       <c r="E23" s="7">
         <f ca="1">IF(E10&gt;Polio!B5,Polio!B5,IF(Scenario_data!E10 &lt;Polio!A5,Polio!A5,Scenario_data!E10))</f>
-        <v>622347907.45734739</v>
+        <v>762464447.93890333</v>
       </c>
       <c r="F23" s="7">
         <f ca="1">IF(F10&gt;Polio!B6,Polio!B6,IF(Scenario_data!F10 &lt;Polio!A6,Polio!A6,Scenario_data!F10))</f>
-        <v>797050394.14084923</v>
+        <v>686389314.4452064</v>
       </c>
       <c r="G23" s="7">
         <f ca="1">IF(G10&gt;Polio!B7,Polio!B7,IF(Scenario_data!G10 &lt;Polio!A7,Polio!A7,Scenario_data!G10))</f>
-        <v>761047792.5542922</v>
+        <v>799985931.68116021</v>
       </c>
       <c r="H23" s="7">
         <f ca="1">IF(H10&gt;Polio!B8,Polio!B8,IF(Scenario_data!H10 &lt;Polio!A8,Polio!A8,Scenario_data!H10))</f>
-        <v>845891380.52937686</v>
+        <v>831863821.14259303</v>
       </c>
       <c r="I23" s="7">
         <f ca="1">IF(I10&gt;Polio!B9,Polio!B9,IF(Scenario_data!I10 &lt;Polio!A9,Polio!A9,Scenario_data!I10))</f>
-        <v>935343794.73410392</v>
+        <v>873350186.74147618</v>
       </c>
       <c r="J23" s="7">
         <f ca="1">IF(J10&gt;Polio!B10,Polio!B10,IF(Scenario_data!J10 &lt;Polio!A10,Polio!A10,Scenario_data!J10))</f>
-        <v>864053553.89152241</v>
+        <v>816658245.66131377</v>
       </c>
       <c r="K23" s="7">
         <f ca="1">IF(K10&gt;Polio!B11,Polio!B11,IF(Scenario_data!K10 &lt;Polio!A11,Polio!A11,Scenario_data!K10))</f>
-        <v>970430798.10298693</v>
+        <v>962728529.51436865</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -4022,43 +4093,43 @@
       </c>
       <c r="B24" s="7">
         <f ca="1">IF(B11&gt;HPV!B2,HPV!B2,IF(Scenario_data!B11 &lt;HPV!A2,HPV!A2,Scenario_data!B11))</f>
-        <v>27360022.551898535</v>
+        <v>31963266.345840931</v>
       </c>
       <c r="C24" s="7">
         <f ca="1">IF(C11&gt;HPV!B3,HPV!B3,IF(Scenario_data!C11 &lt;HPV!A3,HPV!A3,Scenario_data!C11))</f>
-        <v>35671995.023775443</v>
+        <v>37221300.311860926</v>
       </c>
       <c r="D24" s="7">
         <f ca="1">IF(D11&gt;HPV!B4,HPV!B4,IF(Scenario_data!D11 &lt;HPV!A4,HPV!A4,Scenario_data!D11))</f>
-        <v>40957965.06674134</v>
+        <v>40900242.142210245</v>
       </c>
       <c r="E24" s="7">
         <f ca="1">IF(E11&gt;HPV!B5,HPV!B5,IF(Scenario_data!E11 &lt;HPV!A5,HPV!A5,Scenario_data!E11))</f>
-        <v>46651821.38484703</v>
+        <v>46648830.091460817</v>
       </c>
       <c r="F24" s="7">
         <f ca="1">IF(F11&gt;HPV!B6,HPV!B6,IF(Scenario_data!F11 &lt;HPV!A6,HPV!A6,Scenario_data!F11))</f>
-        <v>52037652.38280721</v>
+        <v>51958960.220131822</v>
       </c>
       <c r="G24" s="7">
         <f ca="1">IF(G11&gt;HPV!B7,HPV!B7,IF(Scenario_data!G11 &lt;HPV!A7,HPV!A7,Scenario_data!G11))</f>
-        <v>58485474.245817833</v>
+        <v>55169936.314006709</v>
       </c>
       <c r="H24" s="7">
         <f ca="1">IF(H11&gt;HPV!B8,HPV!B8,IF(Scenario_data!H11 &lt;HPV!A8,HPV!A8,Scenario_data!H11))</f>
-        <v>67839325.216113374</v>
+        <v>67707718.14164719</v>
       </c>
       <c r="I24" s="7">
         <f ca="1">IF(I11&gt;HPV!B9,HPV!B9,IF(Scenario_data!I11 &lt;HPV!A9,HPV!A9,Scenario_data!I11))</f>
-        <v>70647584.994573519</v>
+        <v>72924338.547077373</v>
       </c>
       <c r="J24" s="7">
         <f ca="1">IF(J11&gt;HPV!B10,HPV!B10,IF(Scenario_data!J11 &lt;HPV!A10,HPV!A10,Scenario_data!J11))</f>
-        <v>83688572.811029285</v>
+        <v>82191336.158397973</v>
       </c>
       <c r="K24" s="7">
         <f ca="1">IF(K11&gt;HPV!B11,HPV!B11,IF(Scenario_data!K11 &lt;HPV!A11,HPV!A11,Scenario_data!K11))</f>
-        <v>91343968.710075229</v>
+        <v>90347937.70977132</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -4067,43 +4138,43 @@
       </c>
       <c r="B25" s="7">
         <f ca="1">IF(B12&gt;Rotavirus!B2,Rotavirus!B2,IF(Scenario_data!B12 &lt;Rotavirus!A2,Rotavirus!A2,Scenario_data!B12))</f>
-        <v>205345673.76967528</v>
+        <v>180626332.14641702</v>
       </c>
       <c r="C25" s="7">
         <f ca="1">IF(C12&gt;Rotavirus!B3,Rotavirus!B3,IF(Scenario_data!C12 &lt;Rotavirus!A3,Rotavirus!A3,Scenario_data!C12))</f>
-        <v>190512087.12484357</v>
+        <v>234903455.59618309</v>
       </c>
       <c r="D25" s="7">
         <f ca="1">IF(D12&gt;Rotavirus!B4,Rotavirus!B4,IF(Scenario_data!D12 &lt;Rotavirus!A4,Rotavirus!A4,Scenario_data!D12))</f>
-        <v>267314617.84087193</v>
+        <v>251984068.42984644</v>
       </c>
       <c r="E25" s="7">
         <f ca="1">IF(E12&gt;Rotavirus!B5,Rotavirus!B5,IF(Scenario_data!E12 &lt;Rotavirus!A5,Rotavirus!A5,Scenario_data!E12))</f>
-        <v>247533526.86054593</v>
+        <v>239942103.58603629</v>
       </c>
       <c r="F25" s="7">
         <f ca="1">IF(F12&gt;Rotavirus!B6,Rotavirus!B6,IF(Scenario_data!F12 &lt;Rotavirus!A6,Rotavirus!A6,Scenario_data!F12))</f>
-        <v>328611798.83259988</v>
+        <v>344365641.33358532</v>
       </c>
       <c r="G25" s="7">
         <f ca="1">IF(G12&gt;Rotavirus!B7,Rotavirus!B7,IF(Scenario_data!G12 &lt;Rotavirus!A7,Rotavirus!A7,Scenario_data!G12))</f>
-        <v>369108084.02593571</v>
+        <v>377272561.38604409</v>
       </c>
       <c r="H25" s="7">
         <f ca="1">IF(H12&gt;Rotavirus!B8,Rotavirus!B8,IF(Scenario_data!H12 &lt;Rotavirus!A8,Rotavirus!A8,Scenario_data!H12))</f>
-        <v>438429986.68232673</v>
+        <v>423357966.73157269</v>
       </c>
       <c r="I25" s="7">
         <f ca="1">IF(I12&gt;Rotavirus!B9,Rotavirus!B9,IF(Scenario_data!I12 &lt;Rotavirus!A9,Rotavirus!A9,Scenario_data!I12))</f>
-        <v>507323170.41951501</v>
+        <v>567729050.62302148</v>
       </c>
       <c r="J25" s="7">
         <f ca="1">IF(J12&gt;Rotavirus!B10,Rotavirus!B10,IF(Scenario_data!J12 &lt;Rotavirus!A10,Rotavirus!A10,Scenario_data!J12))</f>
-        <v>594007843.33068144</v>
+        <v>605786630.78349292</v>
       </c>
       <c r="K25" s="7">
         <f ca="1">IF(K12&gt;Rotavirus!B11,Rotavirus!B11,IF(Scenario_data!K12 &lt;Rotavirus!A11,Rotavirus!A11,Scenario_data!K12))</f>
-        <v>731926952.29417491</v>
+        <v>791598901.25984669</v>
       </c>
       <c r="M25" s="4"/>
     </row>
@@ -4113,43 +4184,43 @@
       </c>
       <c r="B26" s="7">
         <f ca="1">IF(B13&gt;PCV!B2,PCV!B2,IF(Scenario_data!B13 &lt;PCV!A2,PCV!A2,Scenario_data!B13))</f>
-        <v>224986828.00133488</v>
+        <v>229617047.20396319</v>
       </c>
       <c r="C26" s="7">
         <f ca="1">IF(C13&gt;PCV!B3,PCV!B3,IF(Scenario_data!C13 &lt;PCV!A3,PCV!A3,Scenario_data!C13))</f>
-        <v>253236124.44606084</v>
+        <v>240945752.67308432</v>
       </c>
       <c r="D26" s="7">
         <f ca="1">IF(D13&gt;PCV!B4,PCV!B4,IF(Scenario_data!D13 &lt;PCV!A4,PCV!A4,Scenario_data!D13))</f>
-        <v>252829865.25797909</v>
+        <v>276233823.85737103</v>
       </c>
       <c r="E26" s="7">
         <f ca="1">IF(E13&gt;PCV!B5,PCV!B5,IF(Scenario_data!E13 &lt;PCV!A5,PCV!A5,Scenario_data!E13))</f>
-        <v>299137152.53839397</v>
+        <v>314594025.93042862</v>
       </c>
       <c r="F26" s="7">
         <f ca="1">IF(F13&gt;PCV!B6,PCV!B6,IF(Scenario_data!F13 &lt;PCV!A6,PCV!A6,Scenario_data!F13))</f>
-        <v>339926643.43062532</v>
+        <v>321897015.9009065</v>
       </c>
       <c r="G26" s="7">
         <f ca="1">IF(G13&gt;PCV!B7,PCV!B7,IF(Scenario_data!G13 &lt;PCV!A7,PCV!A7,Scenario_data!G13))</f>
-        <v>369443410.5810349</v>
+        <v>386260327.82587272</v>
       </c>
       <c r="H26" s="7">
         <f ca="1">IF(H13&gt;PCV!B8,PCV!B8,IF(Scenario_data!H13 &lt;PCV!A8,PCV!A8,Scenario_data!H13))</f>
-        <v>402155465.65981758</v>
+        <v>405501499.43285483</v>
       </c>
       <c r="I26" s="7">
         <f ca="1">IF(I13&gt;PCV!B9,PCV!B9,IF(Scenario_data!I13 &lt;PCV!A9,PCV!A9,Scenario_data!I13))</f>
-        <v>441686216.20688999</v>
+        <v>458134082.10548717</v>
       </c>
       <c r="J26" s="7">
         <f ca="1">IF(J13&gt;PCV!B10,PCV!B10,IF(Scenario_data!J13 &lt;PCV!A10,PCV!A10,Scenario_data!J13))</f>
-        <v>484572073.16770411</v>
+        <v>470477084.71559083</v>
       </c>
       <c r="K26" s="7">
         <f ca="1">IF(K13&gt;PCV!B11,PCV!B11,IF(Scenario_data!K13 &lt;PCV!A11,PCV!A11,Scenario_data!K13))</f>
-        <v>413676643.20716715</v>
+        <v>428131633.6187433</v>
       </c>
       <c r="M26" s="4"/>
     </row>

</xml_diff>

<commit_message>
updated some functions to test MMR only
</commit_message>
<xml_diff>
--- a/DATA/demand/antigen_CI_Random_generator.xlsx
+++ b/DATA/demand/antigen_CI_Random_generator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/demand/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="603" documentId="11_4A5645C871AEA98286DE389EAFF8EF0F542BC54D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74B5E9CD-00B0-4057-8956-E930C6C7739A}"/>
+  <xr:revisionPtr revIDLastSave="619" documentId="11_4A5645C871AEA98286DE389EAFF8EF0F542BC54D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D09D86B8-C7E8-457D-8269-60700EE93632}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-7070" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Diphtheria" sheetId="1" r:id="rId1"/>
@@ -336,34 +336,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>427844524.08335775</c:v>
+                  <c:v>473706567.66978431</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>266493540.45622987</c:v>
+                  <c:v>570594641.52828038</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>690921430.33690572</c:v>
+                  <c:v>585210136.55053055</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>608559229.60524082</c:v>
+                  <c:v>435020009.64618689</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>663849922.05193794</c:v>
+                  <c:v>866602491.50723958</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>720017052.81562459</c:v>
+                  <c:v>623809987.65864646</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>889418994.55034482</c:v>
+                  <c:v>866898844.74215269</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>904042059.50542402</c:v>
+                  <c:v>934709281.9009701</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1015447126.9340428</c:v>
+                  <c:v>947646378.30959857</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>924995113.19309568</c:v>
+                  <c:v>1040074905.1036351</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -408,34 +408,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>32215325.210729256</c:v>
+                  <c:v>23467997.572137151</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45516332.979260825</c:v>
+                  <c:v>35510711.794363424</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>33898087.031309105</c:v>
+                  <c:v>35266359.877763003</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>42814676.437276535</c:v>
+                  <c:v>25446776.697447091</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>36449281.749024712</c:v>
+                  <c:v>30022097.201207686</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>34376475.810845077</c:v>
+                  <c:v>40043367.084398068</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>39757843.010042816</c:v>
+                  <c:v>51191171.492407605</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>49608710.232102938</c:v>
+                  <c:v>53880172.186520286</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>64076046.965096839</c:v>
+                  <c:v>61418555.656488307</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>53151222.967799768</c:v>
+                  <c:v>61868093.835668549</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -480,34 +480,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>321465048.4790833</c:v>
+                  <c:v>420258029.24758023</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>338050229.20354372</c:v>
+                  <c:v>543707292.87605286</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>383103937.96252614</c:v>
+                  <c:v>334695908.16790795</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>566246441.65829504</c:v>
+                  <c:v>519154511.85992396</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>462931671.903368</c:v>
+                  <c:v>510189100.7344588</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>678288191.2504704</c:v>
+                  <c:v>441364812.46718419</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>685059803.96362448</c:v>
+                  <c:v>484364087.70027268</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>481911360.12481743</c:v>
+                  <c:v>597874517.63054919</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>628165183.97071981</c:v>
+                  <c:v>741566200.5050931</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>706453621.3172642</c:v>
+                  <c:v>855874542.56718016</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -552,34 +552,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>625306808.80609596</c:v>
+                  <c:v>713539037.82450485</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>574773030.64024889</c:v>
+                  <c:v>676678971.45618701</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>723594153.53824306</c:v>
+                  <c:v>738393115.67260265</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>840827455.21154118</c:v>
+                  <c:v>990111031.60462713</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>839566408.24645913</c:v>
+                  <c:v>965873400.97549963</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1175682702.2142451</c:v>
+                  <c:v>1080316776.7418959</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1345041665.9302816</c:v>
+                  <c:v>1412563685.8095207</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1635771765.4634292</c:v>
+                  <c:v>1620000372.0732105</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1608781146.4265878</c:v>
+                  <c:v>1491301961.5772977</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1925303189.7746534</c:v>
+                  <c:v>1949799843.1313996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -624,34 +624,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>638898240.21864259</c:v>
+                  <c:v>602611272.63806105</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>645057838.57984638</c:v>
+                  <c:v>679680645.46956027</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>635282685.42925298</c:v>
+                  <c:v>641345167.61468804</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>699956110.31624317</c:v>
+                  <c:v>693797485.51920307</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>709104697.11908937</c:v>
+                  <c:v>735474247.18602145</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>631294572.8514111</c:v>
+                  <c:v>709073886.53999329</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>637984108.1665597</c:v>
+                  <c:v>745903750.12060642</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>667541325.0782249</c:v>
+                  <c:v>706099567.93033385</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>757344004.95768011</c:v>
+                  <c:v>772701541.94441164</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>725685492.89085746</c:v>
+                  <c:v>746531897.50895524</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -696,34 +696,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>315804189.42996383</c:v>
+                  <c:v>344317955.14232874</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>307434632.62051517</c:v>
+                  <c:v>383111201.9068777</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>333184326.93666649</c:v>
+                  <c:v>355296244.24221355</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>359538479.32139218</c:v>
+                  <c:v>354663060.69086301</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>390285709.98276132</c:v>
+                  <c:v>385521449.16832978</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>402564103.74916875</c:v>
+                  <c:v>378709611.29204273</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>377405849.56199503</c:v>
+                  <c:v>393297932.8817426</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>340648666.21157545</c:v>
+                  <c:v>346461994.76831281</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>402285214.5380131</c:v>
+                  <c:v>379199116.50095987</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>417892522.16453439</c:v>
+                  <c:v>391817797.15231961</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -770,34 +770,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>449867903.82097661</c:v>
+                  <c:v>384667427.68182176</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>430976971.81612772</c:v>
+                  <c:v>380976440.78970921</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>421083322.20448852</c:v>
+                  <c:v>419261782.32727981</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>374007214.57592791</c:v>
+                  <c:v>368252251.45383519</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>400135903.70491248</c:v>
+                  <c:v>410413715.83364964</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>407466241.99841297</c:v>
+                  <c:v>433164454.63721949</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>408720007.50686431</c:v>
+                  <c:v>409985741.80634028</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>407827597.23438323</c:v>
+                  <c:v>449734582.26859444</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>349990551.18024623</c:v>
+                  <c:v>404159122.67418867</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>472720841.86251247</c:v>
+                  <c:v>436583036.99487764</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -844,34 +844,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>325602085.99996263</c:v>
+                  <c:v>299798463.44257021</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>317824203.00978869</c:v>
+                  <c:v>299210494.62320864</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>339636905.00294036</c:v>
+                  <c:v>337698872.83373952</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>337903547.41550303</c:v>
+                  <c:v>331646672.76028872</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>360246905.66393006</c:v>
+                  <c:v>347464943.41047776</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>366909200.58424103</c:v>
+                  <c:v>386705921.48365819</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>352892475.03423172</c:v>
+                  <c:v>382836050.02938908</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>398952421.15679967</c:v>
+                  <c:v>387186374.86042023</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>403596167.58389676</c:v>
+                  <c:v>394100921.73965818</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>387444452.78617281</c:v>
+                  <c:v>387291454.13088143</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -918,34 +918,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>716469135.2208643</c:v>
+                  <c:v>652824044.21196711</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>609821971.85227132</c:v>
+                  <c:v>690546743.04875004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>695301475.81519341</c:v>
+                  <c:v>692676867.17088211</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>762464447.93890333</c:v>
+                  <c:v>654861721.33793247</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>686389314.4452064</c:v>
+                  <c:v>700060601.90627897</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>799985931.68116021</c:v>
+                  <c:v>798863703.98095632</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>831863821.14259303</c:v>
+                  <c:v>879720173.04280317</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>873350186.74147618</c:v>
+                  <c:v>887473998.43785214</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>816658245.66131377</c:v>
+                  <c:v>836072319.12820292</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>962728529.51436865</c:v>
+                  <c:v>986116583.99462807</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -992,34 +992,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>31963266.345840931</c:v>
+                  <c:v>30560524.29243347</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37221300.311860926</c:v>
+                  <c:v>34918342.758120202</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40900242.142210245</c:v>
+                  <c:v>41436076.686650589</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>46648830.091460817</c:v>
+                  <c:v>46040942.282288276</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>51958960.220131822</c:v>
+                  <c:v>54828050.269251928</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>55169936.314006709</c:v>
+                  <c:v>57301506.134691209</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67707718.14164719</c:v>
+                  <c:v>68291594.421742514</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>72924338.547077373</c:v>
+                  <c:v>74993654.123364374</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>82191336.158397973</c:v>
+                  <c:v>82144437.209521398</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>90347937.70977132</c:v>
+                  <c:v>90825685.230482191</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1066,34 +1066,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>180626332.14641702</c:v>
+                  <c:v>187657992.33179039</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>234903455.59618309</c:v>
+                  <c:v>225709798.05529684</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>251984068.42984644</c:v>
+                  <c:v>210347798.03823003</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>239942103.58603629</c:v>
+                  <c:v>280408646.42582417</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>344365641.33358532</c:v>
+                  <c:v>309654253.49114066</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>377272561.38604409</c:v>
+                  <c:v>358892927.70832986</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>423357966.73157269</c:v>
+                  <c:v>439328951.17153937</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>567729050.62302148</c:v>
+                  <c:v>540994027.48965824</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>605786630.78349292</c:v>
+                  <c:v>622275062.8185575</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>791598901.25984669</c:v>
+                  <c:v>740001258.35933352</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1140,34 +1140,34 @@
                 <c:formatCode>0.00E+00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>229617047.20396319</c:v>
+                  <c:v>216802553.46174526</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>240945752.67308432</c:v>
+                  <c:v>249520049.08285519</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>276233823.85737103</c:v>
+                  <c:v>281047500.530514</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>314594025.93042862</c:v>
+                  <c:v>319452704.40594953</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>321897015.9009065</c:v>
+                  <c:v>340266975.06073743</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>386260327.82587272</c:v>
+                  <c:v>369787155.59154975</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>405501499.43285483</c:v>
+                  <c:v>410950595.54557264</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>458134082.10548717</c:v>
+                  <c:v>451215498.21884525</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>470477084.71559083</c:v>
+                  <c:v>504019857.09622318</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>428131633.6187433</c:v>
+                  <c:v>424042535.01040512</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1978,6 +1978,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2263,14 +2267,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2284,7 +2289,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>545886518.23867655</v>
       </c>
@@ -2299,8 +2304,9 @@
         <f>(B2-C2)/1.96</f>
         <v>58977087.859632529</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>508228721.08986032</v>
       </c>
@@ -2315,8 +2321,9 @@
         <f t="shared" ref="D3:D11" si="1">(B3-C3)/1.96</f>
         <v>100497668.94220564</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>472845159.87652242</v>
       </c>
@@ -2331,8 +2338,9 @@
         <f t="shared" si="1"/>
         <v>146758824.65147597</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>437709524.92591959</v>
       </c>
@@ -2347,8 +2355,9 @@
         <f t="shared" si="1"/>
         <v>200553151.28297362</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>402698196.9396286</v>
       </c>
@@ -2363,8 +2372,9 @@
         <f t="shared" si="1"/>
         <v>264083490.42320368</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>368115323.15745407</v>
       </c>
@@ -2379,8 +2389,9 @@
         <f t="shared" si="1"/>
         <v>339829561.70663702</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>334354354.94743532</v>
       </c>
@@ -2395,8 +2406,9 @@
         <f t="shared" si="1"/>
         <v>430870881.86331576</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="4"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>301789669.78195262</v>
       </c>
@@ -2411,8 +2423,9 @@
         <f t="shared" si="1"/>
         <v>541139408.8635391</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="4"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>270737783.37456232</v>
       </c>
@@ -2427,8 +2440,9 @@
         <f t="shared" si="1"/>
         <v>675698545.01567936</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="4"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>241444983.2206544</v>
       </c>
@@ -2443,8 +2457,9 @@
         <f t="shared" si="1"/>
         <v>841090339.27080405</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="4"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -2859,7 +2874,7 @@
         <v>31963266.345840931</v>
       </c>
       <c r="C2">
-        <f t="shared" ref="C2:C11" si="0">AVERAGE(A2:B2)</f>
+        <f>AVERAGE(A2:B2)</f>
         <v>28939518.431579627</v>
       </c>
       <c r="D2" s="4">
@@ -2875,7 +2890,7 @@
         <v>39307452.706052743</v>
       </c>
       <c r="C3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C2:C11" si="0">AVERAGE(A3:B3)</f>
         <v>35989921.019888297</v>
       </c>
       <c r="D3" s="4">
@@ -3146,43 +3161,43 @@
       </c>
       <c r="B2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C2,Measles!$D$2)</f>
-        <v>427844524.08335775</v>
+        <v>473706567.66978431</v>
       </c>
       <c r="C2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C3,Measles!$D$2)</f>
-        <v>266493540.45622987</v>
+        <v>570594641.52828038</v>
       </c>
       <c r="D2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C4,Measles!$D$2)</f>
-        <v>690921430.33690572</v>
+        <v>585210136.55053055</v>
       </c>
       <c r="E2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C5,Measles!$D$2)</f>
-        <v>608559229.60524082</v>
+        <v>435020009.64618689</v>
       </c>
       <c r="F2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C6,Measles!$D$2)</f>
-        <v>663849922.05193794</v>
+        <v>866602491.50723958</v>
       </c>
       <c r="G2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C7,Measles!$D$2)</f>
-        <v>720017052.81562459</v>
+        <v>623809987.65864646</v>
       </c>
       <c r="H2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C8,Measles!$D$2)</f>
-        <v>889418994.55034482</v>
+        <v>866898844.74215269</v>
       </c>
       <c r="I2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C9,Measles!$D$2)</f>
-        <v>904042059.50542402</v>
+        <v>934709281.9009701</v>
       </c>
       <c r="J2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C10,Measles!$D$2)</f>
-        <v>1015447126.9340428</v>
+        <v>947646378.30959857</v>
       </c>
       <c r="K2" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Measles!$C11,Measles!$D$2)</f>
-        <v>924995113.19309568</v>
+        <v>1040074905.1036351</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
@@ -3191,43 +3206,43 @@
       </c>
       <c r="B3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C2,Mumps!$D$2)</f>
-        <v>32215325.210729256</v>
+        <v>23467997.572137151</v>
       </c>
       <c r="C3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C3,Mumps!$D$2)</f>
-        <v>45516332.979260825</v>
+        <v>35510711.794363424</v>
       </c>
       <c r="D3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C4,Mumps!$D$2)</f>
-        <v>33898087.031309105</v>
+        <v>35266359.877763003</v>
       </c>
       <c r="E3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C5,Mumps!$D$2)</f>
-        <v>42814676.437276535</v>
+        <v>25446776.697447091</v>
       </c>
       <c r="F3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C6,Mumps!$D$2)</f>
-        <v>36449281.749024712</v>
+        <v>30022097.201207686</v>
       </c>
       <c r="G3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C7,Mumps!$D$2)</f>
-        <v>34376475.810845077</v>
+        <v>40043367.084398068</v>
       </c>
       <c r="H3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C8,Mumps!$D$2)</f>
-        <v>39757843.010042816</v>
+        <v>51191171.492407605</v>
       </c>
       <c r="I3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C9,Mumps!$D$2)</f>
-        <v>49608710.232102938</v>
+        <v>53880172.186520286</v>
       </c>
       <c r="J3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C10,Mumps!$D$2)</f>
-        <v>64076046.965096839</v>
+        <v>61418555.656488307</v>
       </c>
       <c r="K3" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Mumps!$C11,Mumps!$D$2)</f>
-        <v>53151222.967799768</v>
+        <v>61868093.835668549</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -3236,43 +3251,43 @@
       </c>
       <c r="B4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C2,Rubella!$D$2)</f>
-        <v>321465048.4790833</v>
+        <v>420258029.24758023</v>
       </c>
       <c r="C4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C3,Rubella!$D$2)</f>
-        <v>338050229.20354372</v>
+        <v>543707292.87605286</v>
       </c>
       <c r="D4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C4,Rubella!$D$2)</f>
-        <v>383103937.96252614</v>
+        <v>334695908.16790795</v>
       </c>
       <c r="E4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C5,Rubella!$D$2)</f>
-        <v>566246441.65829504</v>
+        <v>519154511.85992396</v>
       </c>
       <c r="F4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C6,Rubella!$D$2)</f>
-        <v>462931671.903368</v>
+        <v>510189100.7344588</v>
       </c>
       <c r="G4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C7,Rubella!$D$2)</f>
-        <v>678288191.2504704</v>
+        <v>441364812.46718419</v>
       </c>
       <c r="H4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C8,Rubella!$D$2)</f>
-        <v>685059803.96362448</v>
+        <v>484364087.70027268</v>
       </c>
       <c r="I4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C9,Rubella!$D$2)</f>
-        <v>481911360.12481743</v>
+        <v>597874517.63054919</v>
       </c>
       <c r="J4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C10,Rubella!$D$2)</f>
-        <v>628165183.97071981</v>
+        <v>741566200.5050931</v>
       </c>
       <c r="K4" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rubella!$C11,Rubella!$D$2)</f>
-        <v>706453621.3172642</v>
+        <v>855874542.56718016</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.25">
@@ -3281,43 +3296,43 @@
       </c>
       <c r="B5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C2,Diphtheria!$D$2)</f>
-        <v>625306808.80609596</v>
+        <v>713539037.82450485</v>
       </c>
       <c r="C5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C3,Diphtheria!$D$2)</f>
-        <v>574773030.64024889</v>
+        <v>676678971.45618701</v>
       </c>
       <c r="D5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C4,Diphtheria!$D$2)</f>
-        <v>723594153.53824306</v>
+        <v>738393115.67260265</v>
       </c>
       <c r="E5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C5,Diphtheria!$D$2)</f>
-        <v>840827455.21154118</v>
+        <v>990111031.60462713</v>
       </c>
       <c r="F5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C6,Diphtheria!$D$2)</f>
-        <v>839566408.24645913</v>
+        <v>965873400.97549963</v>
       </c>
       <c r="G5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C8,Diphtheria!$D$2)</f>
-        <v>1175682702.2142451</v>
+        <v>1080316776.7418959</v>
       </c>
       <c r="H5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C9,Diphtheria!$D$2)</f>
-        <v>1345041665.9302816</v>
+        <v>1412563685.8095207</v>
       </c>
       <c r="I5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1635771765.4634292</v>
+        <v>1620000372.0732105</v>
       </c>
       <c r="J5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C10,Diphtheria!$D$2)</f>
-        <v>1608781146.4265878</v>
+        <v>1491301961.5772977</v>
       </c>
       <c r="K5" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Diphtheria!$C11,Diphtheria!$D$2)</f>
-        <v>1925303189.7746534</v>
+        <v>1949799843.1313996</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.25">
@@ -3326,43 +3341,43 @@
       </c>
       <c r="B6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C2,Tetanus!$D$2)</f>
-        <v>638898240.21864259</v>
+        <v>602611272.63806105</v>
       </c>
       <c r="C6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C3,Tetanus!$D$2)</f>
-        <v>645057838.57984638</v>
+        <v>679680645.46956027</v>
       </c>
       <c r="D6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C4,Tetanus!$D$2)</f>
-        <v>635282685.42925298</v>
+        <v>641345167.61468804</v>
       </c>
       <c r="E6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C5,Tetanus!$D$2)</f>
-        <v>699956110.31624317</v>
+        <v>693797485.51920307</v>
       </c>
       <c r="F6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C6,Tetanus!$D$2)</f>
-        <v>709104697.11908937</v>
+        <v>735474247.18602145</v>
       </c>
       <c r="G6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C7,Tetanus!$D$2)</f>
-        <v>631294572.8514111</v>
+        <v>709073886.53999329</v>
       </c>
       <c r="H6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C8,Tetanus!$D$2)</f>
-        <v>637984108.1665597</v>
+        <v>745903750.12060642</v>
       </c>
       <c r="I6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C9,Tetanus!$D$2)</f>
-        <v>667541325.0782249</v>
+        <v>706099567.93033385</v>
       </c>
       <c r="J6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C10,Tetanus!$D$2)</f>
-        <v>757344004.95768011</v>
+        <v>772701541.94441164</v>
       </c>
       <c r="K6" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Tetanus!$C11,Tetanus!$D$2)</f>
-        <v>725685492.89085746</v>
+        <v>746531897.50895524</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
@@ -3371,43 +3386,43 @@
       </c>
       <c r="B7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>315804189.42996383</v>
+        <v>344317955.14232874</v>
       </c>
       <c r="C7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C2,Pertussis!$D$2)</f>
-        <v>307434632.62051517</v>
+        <v>383111201.9068777</v>
       </c>
       <c r="D7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C4,Pertussis!$D$2)</f>
-        <v>333184326.93666649</v>
+        <v>355296244.24221355</v>
       </c>
       <c r="E7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C5,Pertussis!$D$2)</f>
-        <v>359538479.32139218</v>
+        <v>354663060.69086301</v>
       </c>
       <c r="F7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C6,Pertussis!$D$2)</f>
-        <v>390285709.98276132</v>
+        <v>385521449.16832978</v>
       </c>
       <c r="G7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C7,Pertussis!$D$2)</f>
-        <v>402564103.74916875</v>
+        <v>378709611.29204273</v>
       </c>
       <c r="H7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C8,Pertussis!$D$2)</f>
-        <v>377405849.56199503</v>
+        <v>393297932.8817426</v>
       </c>
       <c r="I7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C9,Pertussis!$D$2)</f>
-        <v>340648666.21157545</v>
+        <v>346461994.76831281</v>
       </c>
       <c r="J7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C10,Pertussis!$D$2)</f>
-        <v>402285214.5380131</v>
+        <v>379199116.50095987</v>
       </c>
       <c r="K7" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Pertussis!$C11,Pertussis!$D$2)</f>
-        <v>417892522.16453439</v>
+        <v>391817797.15231961</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.25">
@@ -3416,43 +3431,43 @@
       </c>
       <c r="B8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C2,Hepatitis_B!$D$2)</f>
-        <v>457483356.99579835</v>
+        <v>384667427.68182176</v>
       </c>
       <c r="C8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C3,Hepatitis_B!$D$2)</f>
-        <v>430976971.81612772</v>
+        <v>380976440.78970921</v>
       </c>
       <c r="D8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C4,Hepatitis_B!$D$2)</f>
-        <v>421083322.20448852</v>
+        <v>419261782.32727981</v>
       </c>
       <c r="E8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C5,Hepatitis_B!$D$2)</f>
-        <v>374007214.57592791</v>
+        <v>368252251.45383519</v>
       </c>
       <c r="F8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C6,Hepatitis_B!$D$2)</f>
-        <v>400135903.70491248</v>
+        <v>410413715.83364964</v>
       </c>
       <c r="G8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C7,Hepatitis_B!$D$2)</f>
-        <v>407466241.99841297</v>
+        <v>433164454.63721949</v>
       </c>
       <c r="H8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C8,Hepatitis_B!$D$2)</f>
-        <v>408720007.50686431</v>
+        <v>409985741.80634028</v>
       </c>
       <c r="I8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C9,Hepatitis_B!$D$2)</f>
-        <v>407827597.23438323</v>
+        <v>449734582.26859444</v>
       </c>
       <c r="J8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C10,Hepatitis_B!$D$2)</f>
-        <v>349990551.18024623</v>
+        <v>404159122.67418867</v>
       </c>
       <c r="K8" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,Hepatitis_B!$D$2)</f>
-        <v>472720841.86251247</v>
+        <v>436583036.99487764</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
@@ -3461,43 +3476,43 @@
       </c>
       <c r="B9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C2,Hib!$D$2)</f>
-        <v>325602085.99996263</v>
+        <v>299798463.44257021</v>
       </c>
       <c r="C9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C3,Hib!$D$2)</f>
-        <v>317824203.00978869</v>
+        <v>299210494.62320864</v>
       </c>
       <c r="D9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C4,Hib!$D$2)</f>
-        <v>339636905.00294036</v>
+        <v>337698872.83373952</v>
       </c>
       <c r="E9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C5,Hib!$D$2)</f>
-        <v>337903547.41550303</v>
+        <v>331646672.76028872</v>
       </c>
       <c r="F9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C6,Hib!$D$2)</f>
-        <v>360246905.66393006</v>
+        <v>347464943.41047776</v>
       </c>
       <c r="G9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C7,Hib!$D$2)</f>
-        <v>366909200.58424103</v>
+        <v>386705921.48365819</v>
       </c>
       <c r="H9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C8,Hib!$D$2)</f>
-        <v>352892475.03423172</v>
+        <v>382836050.02938908</v>
       </c>
       <c r="I9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C9,Hib!$D$2)</f>
-        <v>398952421.15679967</v>
+        <v>387186374.86042023</v>
       </c>
       <c r="J9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C10,Hib!$D$2)</f>
-        <v>403596167.58389676</v>
+        <v>394100921.73965818</v>
       </c>
       <c r="K9" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hib!$C11,Hib!$D$2)</f>
-        <v>387444452.78617281</v>
+        <v>387291454.13088143</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
@@ -3506,43 +3521,43 @@
       </c>
       <c r="B10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C2,Polio!$D$2)</f>
-        <v>736527737.92395699</v>
+        <v>652824044.21196711</v>
       </c>
       <c r="C10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C3,Polio!$D$2)</f>
-        <v>609821971.85227132</v>
+        <v>690546743.04875004</v>
       </c>
       <c r="D10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C4,Polio!$D$2)</f>
-        <v>695301475.81519341</v>
+        <v>692676867.17088211</v>
       </c>
       <c r="E10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C5,Polio!$D$2)</f>
-        <v>762464447.93890333</v>
+        <v>654861721.33793247</v>
       </c>
       <c r="F10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C6,Polio!$D$2)</f>
-        <v>686389314.4452064</v>
+        <v>700060601.90627897</v>
       </c>
       <c r="G10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C7,Polio!$D$2)</f>
-        <v>799985931.68116021</v>
+        <v>798863703.98095632</v>
       </c>
       <c r="H10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C8,Polio!$D$2)</f>
-        <v>831863821.14259303</v>
+        <v>879720173.04280317</v>
       </c>
       <c r="I10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C9,Polio!$D$2)</f>
-        <v>873350186.74147618</v>
+        <v>887473998.43785214</v>
       </c>
       <c r="J10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C10,Polio!$D$2)</f>
-        <v>816658245.66131377</v>
+        <v>836072319.12820292</v>
       </c>
       <c r="K10" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Polio!$C11,Polio!$D$2)</f>
-        <v>962728529.51436865</v>
+        <v>986116583.99462807</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.25">
@@ -3551,43 +3566,43 @@
       </c>
       <c r="B11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C2,HPV!$D$2)</f>
-        <v>32323300.612997241</v>
+        <v>30560524.29243347</v>
       </c>
       <c r="C11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C3,HPV!$D$2)</f>
-        <v>37221300.311860926</v>
+        <v>34918342.758120202</v>
       </c>
       <c r="D11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C4,HPV!$D$2)</f>
-        <v>40900242.142210245</v>
+        <v>41436076.686650589</v>
       </c>
       <c r="E11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C5,HPV!$D$2)</f>
-        <v>46648830.091460817</v>
+        <v>46040942.282288276</v>
       </c>
       <c r="F11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C6,HPV!$D$2)</f>
-        <v>51958960.220131822</v>
+        <v>54828050.269251928</v>
       </c>
       <c r="G11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C7,HPV!$D$2)</f>
-        <v>55169936.314006709</v>
+        <v>57301506.134691209</v>
       </c>
       <c r="H11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C8,HPV!$D$2)</f>
-        <v>67707718.14164719</v>
+        <v>68291594.421742514</v>
       </c>
       <c r="I11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C9,HPV!$D$2)</f>
-        <v>72924338.547077373</v>
+        <v>74993654.123364374</v>
       </c>
       <c r="J11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C10,HPV!$D$2)</f>
-        <v>82191336.158397973</v>
+        <v>82144437.209521398</v>
       </c>
       <c r="K11" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),HPV!$C11,HPV!$D$2)</f>
-        <v>90347937.70977132</v>
+        <v>90825685.230482191</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.25">
@@ -3596,43 +3611,43 @@
       </c>
       <c r="B12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C2,Rotavirus!$D$2)</f>
-        <v>180626332.14641702</v>
+        <v>187657992.33179039</v>
       </c>
       <c r="C12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C3,Rotavirus!$D$2)</f>
-        <v>234903455.59618309</v>
+        <v>225709798.05529684</v>
       </c>
       <c r="D12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C4,Rotavirus!$D$2)</f>
-        <v>251984068.42984644</v>
+        <v>210347798.03823003</v>
       </c>
       <c r="E12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C5,Rotavirus!$D$2)</f>
-        <v>239942103.58603629</v>
+        <v>280408646.42582417</v>
       </c>
       <c r="F12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C6,Rotavirus!$D$2)</f>
-        <v>344365641.33358532</v>
+        <v>309654253.49114066</v>
       </c>
       <c r="G12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C7,Rotavirus!$D$2)</f>
-        <v>377272561.38604409</v>
+        <v>358892927.70832986</v>
       </c>
       <c r="H12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C8,Rotavirus!$D$2)</f>
-        <v>423357966.73157269</v>
+        <v>439328951.17153937</v>
       </c>
       <c r="I12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C9,Rotavirus!$D$2)</f>
-        <v>567729050.62302148</v>
+        <v>540994027.48965824</v>
       </c>
       <c r="J12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C10,Rotavirus!$D$2)</f>
-        <v>605786630.78349292</v>
+        <v>622275062.8185575</v>
       </c>
       <c r="K12" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Rotavirus!$C11,Rotavirus!$D$2)</f>
-        <v>791598901.25984669</v>
+        <v>740001258.35933352</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.25">
@@ -3641,43 +3656,43 @@
       </c>
       <c r="B13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C2,PCV!$D$2)</f>
-        <v>229617047.20396319</v>
+        <v>216802553.46174526</v>
       </c>
       <c r="C13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C3,PCV!$D$2)</f>
-        <v>240945752.67308432</v>
+        <v>249520049.08285519</v>
       </c>
       <c r="D13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C4,PCV!$D$2)</f>
-        <v>276233823.85737103</v>
+        <v>281047500.530514</v>
       </c>
       <c r="E13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C5,PCV!$D$2)</f>
-        <v>314594025.93042862</v>
+        <v>319452704.40594953</v>
       </c>
       <c r="F13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C6,PCV!$D$2)</f>
-        <v>321897015.9009065</v>
+        <v>340266975.06073743</v>
       </c>
       <c r="G13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C7,PCV!$D$2)</f>
-        <v>386260327.82587272</v>
+        <v>369787155.59154975</v>
       </c>
       <c r="H13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C8,PCV!$D$2)</f>
-        <v>405501499.43285483</v>
+        <v>410950595.54557264</v>
       </c>
       <c r="I13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C9,PCV!$D$2)</f>
-        <v>458134082.10548717</v>
+        <v>451215498.21884525</v>
       </c>
       <c r="J13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),PCV!$C10,PCV!$D$2)</f>
-        <v>470477084.71559083</v>
+        <v>504019857.09622318</v>
       </c>
       <c r="K13" s="4">
         <f ca="1">_xlfn.NORM.INV(RAND(),Hepatitis_B!$C11,PCV!$D$2)</f>
-        <v>428131633.6187433</v>
+        <v>424042535.01040512</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.25">
@@ -3686,43 +3701,43 @@
       </c>
       <c r="B15" s="7">
         <f ca="1">IF(B2&gt;Measles!B2,Measles!B2,IF(Scenario_data!B2 &lt;Measles!A2,Measles!A2,Scenario_data!B2))</f>
-        <v>427844524.08335775</v>
+        <v>473706567.66978431</v>
       </c>
       <c r="C15" s="7">
         <f ca="1">IF(C2&gt;Measles!B3,Measles!B3,IF(Scenario_data!C2 &lt;Measles!A3,Measles!A3,Scenario_data!C2))</f>
-        <v>266493540.45622987</v>
+        <v>570594641.52828038</v>
       </c>
       <c r="D15" s="7">
         <f ca="1">IF(D2&gt;Measles!B4,Measles!B4,IF(Scenario_data!D2 &lt;Measles!A4,Measles!A4,Scenario_data!D2))</f>
-        <v>690921430.33690572</v>
+        <v>585210136.55053055</v>
       </c>
       <c r="E15" s="7">
         <f ca="1">IF(E2&gt;Measles!B5,Measles!B5,IF(Scenario_data!E2 &lt;Measles!A5,Measles!A5,Scenario_data!E2))</f>
-        <v>608559229.60524082</v>
+        <v>435020009.64618689</v>
       </c>
       <c r="F15" s="7">
         <f ca="1">IF(F2&gt;Measles!B6,Measles!B6,IF(Scenario_data!F2 &lt;Measles!A6,Measles!A6,Scenario_data!F2))</f>
-        <v>663849922.05193794</v>
+        <v>866602491.50723958</v>
       </c>
       <c r="G15" s="7">
         <f ca="1">IF(G2&gt;Measles!B7,Measles!B7,IF(Scenario_data!G2 &lt;Measles!A7,Measles!A7,Scenario_data!G2))</f>
-        <v>720017052.81562459</v>
+        <v>623809987.65864646</v>
       </c>
       <c r="H15" s="7">
         <f ca="1">IF(H2&gt;Measles!B8,Measles!B8,IF(Scenario_data!H2 &lt;Measles!A8,Measles!A8,Scenario_data!H2))</f>
-        <v>889418994.55034482</v>
+        <v>866898844.74215269</v>
       </c>
       <c r="I15" s="7">
         <f ca="1">IF(I2&gt;Measles!B9,Measles!B9,IF(Scenario_data!I2 &lt;Measles!A9,Measles!A9,Scenario_data!I2))</f>
-        <v>904042059.50542402</v>
+        <v>934709281.9009701</v>
       </c>
       <c r="J15" s="7">
         <f ca="1">IF(J2&gt;Measles!B10,Measles!B10,IF(Scenario_data!J2 &lt;Measles!A10,Measles!A10,Scenario_data!J2))</f>
-        <v>1015447126.9340428</v>
+        <v>947646378.30959857</v>
       </c>
       <c r="K15" s="7">
         <f ca="1">IF(K2&gt;Measles!B11,Measles!B11,IF(Scenario_data!K2 &lt;Measles!A11,Measles!A11,Scenario_data!K2))</f>
-        <v>924995113.19309568</v>
+        <v>1040074905.1036351</v>
       </c>
       <c r="W15" s="4"/>
       <c r="X15" s="4"/>
@@ -3733,43 +3748,43 @@
       </c>
       <c r="B16" s="7">
         <f ca="1">IF(B3&gt;Mumps!B2,Mumps!B2,IF(Scenario_data!B3 &lt;Mumps!A2,Mumps!A2,Scenario_data!B3))</f>
-        <v>32215325.210729256</v>
+        <v>23467997.572137151</v>
       </c>
       <c r="C16" s="7">
         <f ca="1">IF(C3&gt;Mumps!B3,Mumps!B3,IF(Scenario_data!C3 &lt;Mumps!A3,Mumps!A3,Scenario_data!C3))</f>
-        <v>45516332.979260825</v>
+        <v>35510711.794363424</v>
       </c>
       <c r="D16" s="7">
         <f ca="1">IF(D3&gt;Mumps!B4,Mumps!B4,IF(Scenario_data!D3 &lt;Mumps!A4,Mumps!A4,Scenario_data!D3))</f>
-        <v>33898087.031309105</v>
+        <v>35266359.877763003</v>
       </c>
       <c r="E16" s="7">
         <f ca="1">IF(E3&gt;Mumps!B5,Mumps!B5,IF(Scenario_data!E3 &lt;Mumps!A5,Mumps!A5,Scenario_data!E3))</f>
-        <v>42814676.437276535</v>
+        <v>25446776.697447091</v>
       </c>
       <c r="F16" s="7">
         <f ca="1">IF(F3&gt;Mumps!B6,Mumps!B6,IF(Scenario_data!F3 &lt;Mumps!A6,Mumps!A6,Scenario_data!F3))</f>
-        <v>36449281.749024712</v>
+        <v>30022097.201207686</v>
       </c>
       <c r="G16" s="7">
         <f ca="1">IF(G3&gt;Mumps!B7,Mumps!B7,IF(Scenario_data!G3 &lt;Mumps!A7,Mumps!A7,Scenario_data!G3))</f>
-        <v>34376475.810845077</v>
+        <v>40043367.084398068</v>
       </c>
       <c r="H16" s="7">
         <f ca="1">IF(H3&gt;Mumps!B8,Mumps!B8,IF(Scenario_data!H3 &lt;Mumps!A8,Mumps!A8,Scenario_data!H3))</f>
-        <v>39757843.010042816</v>
+        <v>51191171.492407605</v>
       </c>
       <c r="I16" s="7">
         <f ca="1">IF(I3&gt;Mumps!B9,Mumps!B9,IF(Scenario_data!I3 &lt;Mumps!A9,Mumps!A9,Scenario_data!I3))</f>
-        <v>49608710.232102938</v>
+        <v>53880172.186520286</v>
       </c>
       <c r="J16" s="7">
         <f ca="1">IF(J3&gt;Mumps!B10,Mumps!B10,IF(Scenario_data!J3 &lt;Mumps!A10,Mumps!A10,Scenario_data!J3))</f>
-        <v>64076046.965096839</v>
+        <v>61418555.656488307</v>
       </c>
       <c r="K16" s="7">
         <f ca="1">IF(K3&gt;Mumps!B11,Mumps!B11,IF(Scenario_data!K3 &lt;Mumps!A11,Mumps!A11,Scenario_data!K3))</f>
-        <v>53151222.967799768</v>
+        <v>61868093.835668549</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -3778,43 +3793,43 @@
       </c>
       <c r="B17" s="7">
         <f ca="1">IF(B4&gt;Rubella!B2,Rubella!B2,IF(Scenario_data!B4 &lt;Rubella!A2,Rubella!A2,Scenario_data!B4))</f>
-        <v>321465048.4790833</v>
+        <v>420258029.24758023</v>
       </c>
       <c r="C17" s="7">
         <f ca="1">IF(C4&gt;Rubella!B3,Rubella!B3,IF(Scenario_data!C4 &lt;Rubella!A3,Rubella!A3,Scenario_data!C4))</f>
-        <v>338050229.20354372</v>
+        <v>543707292.87605286</v>
       </c>
       <c r="D17" s="7">
         <f ca="1">IF(D4&gt;Rubella!B4,Rubella!B4,IF(Scenario_data!D4 &lt;Rubella!A4,Rubella!A4,Scenario_data!D4))</f>
-        <v>383103937.96252614</v>
+        <v>334695908.16790795</v>
       </c>
       <c r="E17" s="7">
         <f ca="1">IF(E4&gt;Rubella!B5,Rubella!B5,IF(Scenario_data!E4 &lt;Rubella!A5,Rubella!A5,Scenario_data!E4))</f>
-        <v>566246441.65829504</v>
+        <v>519154511.85992396</v>
       </c>
       <c r="F17" s="7">
         <f ca="1">IF(F4&gt;Rubella!B6,Rubella!B6,IF(Scenario_data!F4 &lt;Rubella!A6,Rubella!A6,Scenario_data!F4))</f>
-        <v>462931671.903368</v>
+        <v>510189100.7344588</v>
       </c>
       <c r="G17" s="7">
         <f ca="1">IF(G4&gt;Rubella!B7,Rubella!B7,IF(Scenario_data!G4 &lt;Rubella!A7,Rubella!A7,Scenario_data!G4))</f>
-        <v>678288191.2504704</v>
+        <v>441364812.46718419</v>
       </c>
       <c r="H17" s="7">
         <f ca="1">IF(H4&gt;Rubella!B8,Rubella!B8,IF(Scenario_data!H4 &lt;Rubella!A8,Rubella!A8,Scenario_data!H4))</f>
-        <v>685059803.96362448</v>
+        <v>484364087.70027268</v>
       </c>
       <c r="I17" s="7">
         <f ca="1">IF(I4&gt;Rubella!B9,Rubella!B9,IF(Scenario_data!I4 &lt;Rubella!A9,Rubella!A9,Scenario_data!I4))</f>
-        <v>481911360.12481743</v>
+        <v>597874517.63054919</v>
       </c>
       <c r="J17" s="7">
         <f ca="1">IF(J4&gt;Rubella!B10,Rubella!B10,IF(Scenario_data!J4 &lt;Rubella!A10,Rubella!A10,Scenario_data!J4))</f>
-        <v>628165183.97071981</v>
+        <v>741566200.5050931</v>
       </c>
       <c r="K17" s="7">
         <f ca="1">IF(K4&gt;Rubella!B12=1,Rubella!B11,IF(Scenario_data!K4 &lt;Rubella!A11,Rubella!A11,Scenario_data!K4))</f>
-        <v>706453621.3172642</v>
+        <v>855874542.56718016</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -3823,43 +3838,43 @@
       </c>
       <c r="B18" s="7">
         <f ca="1">IF(B5&gt;Diphtheria!B2,Diphtheria!B2,IF(Scenario_data!B5 &lt;Diphtheria!A2,Diphtheria!A2,Scenario_data!B5))</f>
-        <v>625306808.80609596</v>
+        <v>713539037.82450485</v>
       </c>
       <c r="C18" s="7">
         <f ca="1">IF(C5&gt;Diphtheria!B3,Diphtheria!B3,IF(Scenario_data!C5 &lt;Diphtheria!A3,Diphtheria!A3,Scenario_data!C5))</f>
-        <v>574773030.64024889</v>
+        <v>676678971.45618701</v>
       </c>
       <c r="D18" s="7">
         <f ca="1">IF(D5&gt;Diphtheria!B4,Diphtheria!B4,IF(Scenario_data!D5 &lt;Diphtheria!A4,Diphtheria!A4,Scenario_data!D5))</f>
-        <v>723594153.53824306</v>
+        <v>738393115.67260265</v>
       </c>
       <c r="E18" s="7">
         <f ca="1">IF(E5&gt;Diphtheria!B5,Diphtheria!B5,IF(Scenario_data!E5 &lt;Diphtheria!A5,Diphtheria!A5,Scenario_data!E5))</f>
-        <v>840827455.21154118</v>
+        <v>990111031.60462713</v>
       </c>
       <c r="F18" s="7">
         <f ca="1">IF(F5&gt;Diphtheria!B6,Diphtheria!B6,IF(Scenario_data!F5 &lt;Diphtheria!A6,Diphtheria!A6,Scenario_data!F5))</f>
-        <v>839566408.24645913</v>
+        <v>965873400.97549963</v>
       </c>
       <c r="G18" s="7">
         <f ca="1">IF(G5&gt;Diphtheria!B7,Diphtheria!B7,IF(Scenario_data!G5 &lt;Diphtheria!A7,Diphtheria!A7,Scenario_data!G5))</f>
-        <v>1175682702.2142451</v>
+        <v>1080316776.7418959</v>
       </c>
       <c r="H18" s="7">
         <f ca="1">IF(H5&gt;Diphtheria!B8,Diphtheria!B8,IF(Scenario_data!H5 &lt;Diphtheria!A8,Diphtheria!A8,Scenario_data!H5))</f>
-        <v>1345041665.9302816</v>
+        <v>1412563685.8095207</v>
       </c>
       <c r="I18" s="7">
         <f ca="1">IF(I5&gt;Diphtheria!B9,Diphtheria!B9,IF(Scenario_data!I5 &lt;Diphtheria!A9,Diphtheria!A9,Scenario_data!I5))</f>
-        <v>1635771765.4634292</v>
+        <v>1620000372.0732105</v>
       </c>
       <c r="J18" s="7">
         <f ca="1">IF(J5&gt;Diphtheria!B10,Diphtheria!B10,IF(Scenario_data!J5 &lt;Diphtheria!A10,Diphtheria!A10,Scenario_data!J5))</f>
-        <v>1608781146.4265878</v>
+        <v>1491301961.5772977</v>
       </c>
       <c r="K18" s="7">
         <f ca="1">IF(K5&gt;Diphtheria!B11,Diphtheria!B11,IF(Scenario_data!K5 &lt;Diphtheria!A11,Diphtheria!A11,Scenario_data!K5))</f>
-        <v>1925303189.7746534</v>
+        <v>1949799843.1313996</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -3868,43 +3883,43 @@
       </c>
       <c r="B19" s="7">
         <f ca="1">IF(B6&gt;Tetanus!B2,Tetanus!B2,IF(Scenario_data!B6 &lt;Tetanus!A2,Tetanus!A2,Scenario_data!B6))</f>
-        <v>638898240.21864259</v>
+        <v>602611272.63806105</v>
       </c>
       <c r="C19" s="7">
         <f ca="1">IF(C6&gt;Tetanus!B3,Tetanus!B3,IF(Scenario_data!C6 &lt;Tetanus!A3,Tetanus!A3,Scenario_data!C6))</f>
-        <v>645057838.57984638</v>
+        <v>679680645.46956027</v>
       </c>
       <c r="D19" s="7">
         <f ca="1">IF(D6&gt;Tetanus!B4,Tetanus!B4,IF(Scenario_data!D6 &lt;Tetanus!A4,Tetanus!A4,Scenario_data!D6))</f>
-        <v>635282685.42925298</v>
+        <v>641345167.61468804</v>
       </c>
       <c r="E19" s="7">
         <f ca="1">IF(E6&gt;Tetanus!B5,Tetanus!B5,IF(Scenario_data!E6 &lt;Tetanus!A5,Tetanus!A5,Scenario_data!E6))</f>
-        <v>699956110.31624317</v>
+        <v>693797485.51920307</v>
       </c>
       <c r="F19" s="7">
         <f ca="1">IF(F6&gt;Tetanus!B6,Tetanus!B6,IF(Scenario_data!F6 &lt;Tetanus!A6,Tetanus!A6,Scenario_data!F6))</f>
-        <v>709104697.11908937</v>
+        <v>735474247.18602145</v>
       </c>
       <c r="G19" s="7">
         <f ca="1">IF(G6&gt;Tetanus!B7,Tetanus!B7,IF(Scenario_data!G6 &lt;Tetanus!A7,Tetanus!A7,Scenario_data!G6))</f>
-        <v>631294572.8514111</v>
+        <v>709073886.53999329</v>
       </c>
       <c r="H19" s="7">
         <f ca="1">IF(H6&gt;Tetanus!B8,Tetanus!B8,IF(Scenario_data!H6 &lt;Tetanus!A8,Tetanus!A8,Scenario_data!H6))</f>
-        <v>637984108.1665597</v>
+        <v>745903750.12060642</v>
       </c>
       <c r="I19" s="7">
         <f ca="1">IF(I6&gt;Tetanus!B9,Tetanus!B9,IF(Scenario_data!I6 &lt;Tetanus!A9,Tetanus!A9,Scenario_data!I6))</f>
-        <v>667541325.0782249</v>
+        <v>706099567.93033385</v>
       </c>
       <c r="J19" s="7">
         <f ca="1">IF(J6&gt;Tetanus!B10,Tetanus!B10,IF(Scenario_data!J6 &lt;Tetanus!A10,Tetanus!A10,Scenario_data!J6))</f>
-        <v>757344004.95768011</v>
+        <v>772701541.94441164</v>
       </c>
       <c r="K19" s="7">
         <f ca="1">IF(K6&gt;Tetanus!B11,Tetanus!B11,IF(Scenario_data!K6 &lt;Tetanus!A11,Tetanus!A11,Scenario_data!K6))</f>
-        <v>725685492.89085746</v>
+        <v>746531897.50895524</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
@@ -3913,43 +3928,43 @@
       </c>
       <c r="B20" s="7">
         <f ca="1">IF(B7&gt;Pertussis!B2,Pertussis!B2,IF(Scenario_data!B7 &lt;Pertussis!A2,Pertussis!A2,Scenario_data!B7))</f>
-        <v>315804189.42996383</v>
+        <v>344317955.14232874</v>
       </c>
       <c r="C20" s="7">
         <f ca="1">IF(C7&gt;Pertussis!B3,Pertussis!B3,IF(Scenario_data!C7 &lt;Pertussis!A3,Pertussis!A3,Scenario_data!C7))</f>
-        <v>307434632.62051517</v>
+        <v>383111201.9068777</v>
       </c>
       <c r="D20" s="7">
         <f ca="1">IF(D7&gt;Pertussis!B4,Pertussis!B4,IF(Scenario_data!D7 &lt;Pertussis!A4,Pertussis!A4,Scenario_data!D7))</f>
-        <v>333184326.93666649</v>
+        <v>355296244.24221355</v>
       </c>
       <c r="E20" s="7">
         <f ca="1">IF(E7&gt;Pertussis!B5,Pertussis!B5,IF(Scenario_data!E7 &lt;Pertussis!A5,Pertussis!A5,Scenario_data!E7))</f>
-        <v>359538479.32139218</v>
+        <v>354663060.69086301</v>
       </c>
       <c r="F20" s="7">
         <f ca="1">IF(F7&gt;Pertussis!B6,Pertussis!B6,IF(Scenario_data!F7 &lt;Pertussis!A6,Pertussis!A6,Scenario_data!F7))</f>
-        <v>390285709.98276132</v>
+        <v>385521449.16832978</v>
       </c>
       <c r="G20" s="7">
         <f ca="1">IF(G7&gt;Pertussis!B7,Pertussis!B7,IF(Scenario_data!G7 &lt;Pertussis!A7,Pertussis!A7,Scenario_data!G7))</f>
-        <v>402564103.74916875</v>
+        <v>378709611.29204273</v>
       </c>
       <c r="H20" s="7">
         <f ca="1">IF(H7&gt;Pertussis!B8,Pertussis!B8,IF(Scenario_data!H7 &lt;Pertussis!A8,Pertussis!A8,Scenario_data!H7))</f>
-        <v>377405849.56199503</v>
+        <v>393297932.8817426</v>
       </c>
       <c r="I20" s="7">
         <f ca="1">IF(I7&gt;Pertussis!B9,Pertussis!B9,IF(Scenario_data!I7 &lt;Pertussis!A9,Pertussis!A9,Scenario_data!I7))</f>
-        <v>340648666.21157545</v>
+        <v>346461994.76831281</v>
       </c>
       <c r="J20" s="7">
         <f ca="1">IF(J7&gt;Pertussis!B10,Pertussis!B10,IF(Scenario_data!J7 &lt;Pertussis!A10,Pertussis!A10,Scenario_data!J7))</f>
-        <v>402285214.5380131</v>
+        <v>379199116.50095987</v>
       </c>
       <c r="K20" s="7">
         <f ca="1">IF(K7&gt;Pertussis!B11,Pertussis!B11,IF(Scenario_data!K7 &lt;Pertussis!A11,Pertussis!A11,Scenario_data!K7))</f>
-        <v>417892522.16453439</v>
+        <v>391817797.15231961</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -3958,43 +3973,43 @@
       </c>
       <c r="B21" s="7">
         <f ca="1">IF(B8&gt;Hepatitis_B!B2,Hepatitis_B!B2,IF(Scenario_data!B8 &lt;Hepatitis_B!A2,Hepatitis_B!A2,Scenario_data!B8))</f>
-        <v>449867903.82097661</v>
+        <v>384667427.68182176</v>
       </c>
       <c r="C21" s="7">
         <f ca="1">IF(C8&gt;Hepatitis_B!B3,Hepatitis_B!B3,IF(Scenario_data!C8 &lt;Hepatitis_B!A3,Hepatitis_B!A3,Scenario_data!C8))</f>
-        <v>430976971.81612772</v>
+        <v>380976440.78970921</v>
       </c>
       <c r="D21" s="7">
         <f ca="1">IF(D8&gt;Hepatitis_B!B4,Hepatitis_B!B4,IF(Scenario_data!D8 &lt;Hepatitis_B!A4,Hepatitis_B!A4,Scenario_data!D8))</f>
-        <v>421083322.20448852</v>
+        <v>419261782.32727981</v>
       </c>
       <c r="E21" s="7">
         <f ca="1">IF(E8&gt;Hepatitis_B!B5,Hepatitis_B!B5,IF(Scenario_data!E8 &lt;Hepatitis_B!A5,Hepatitis_B!A5,Scenario_data!E8))</f>
-        <v>374007214.57592791</v>
+        <v>368252251.45383519</v>
       </c>
       <c r="F21" s="7">
         <f ca="1">IF(F8&gt;Hepatitis_B!B6,Hepatitis_B!B6,IF(Scenario_data!F8 &lt;Hepatitis_B!A6,Hepatitis_B!A6,Scenario_data!F8))</f>
-        <v>400135903.70491248</v>
+        <v>410413715.83364964</v>
       </c>
       <c r="G21" s="7">
         <f ca="1">IF(G8&gt;Hepatitis_B!B7,Hepatitis_B!B7,IF(Scenario_data!G8 &lt;Hepatitis_B!A7,Hepatitis_B!A7,Scenario_data!G8))</f>
-        <v>407466241.99841297</v>
+        <v>433164454.63721949</v>
       </c>
       <c r="H21" s="7">
         <f ca="1">IF(H8&gt;Hepatitis_B!B8,Hepatitis_B!B8,IF(Scenario_data!H8 &lt;Hepatitis_B!A8,Hepatitis_B!A8,Scenario_data!H8))</f>
-        <v>408720007.50686431</v>
+        <v>409985741.80634028</v>
       </c>
       <c r="I21" s="7">
         <f ca="1">IF(I8&gt;Hepatitis_B!B9,Hepatitis_B!B9,IF(Scenario_data!I8 &lt;Hepatitis_B!A9,Hepatitis_B!A9,Scenario_data!I8))</f>
-        <v>407827597.23438323</v>
+        <v>449734582.26859444</v>
       </c>
       <c r="J21" s="7">
         <f ca="1">IF(J8&gt;Hepatitis_B!B10,Hepatitis_B!B10,IF(Scenario_data!J8 &lt;Hepatitis_B!A10,Hepatitis_B!A10,Scenario_data!J8))</f>
-        <v>349990551.18024623</v>
+        <v>404159122.67418867</v>
       </c>
       <c r="K21" s="7">
         <f ca="1">IF(K8&gt;Hepatitis_B!B11,Hepatitis_B!B11,IF(Scenario_data!K8 &lt;Hepatitis_B!A11,Hepatitis_B!A11,Scenario_data!K8))</f>
-        <v>472720841.86251247</v>
+        <v>436583036.99487764</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
@@ -4003,43 +4018,43 @@
       </c>
       <c r="B22" s="7">
         <f ca="1">IF(B9&gt;Hib!B2,Hib!B2,IF(Scenario_data!B9 &lt;Hib!A2,Hib!A2,Scenario_data!B9))</f>
-        <v>325602085.99996263</v>
+        <v>299798463.44257021</v>
       </c>
       <c r="C22" s="7">
         <f ca="1">IF(C9&gt;Hib!B3,Hib!B3,IF(Scenario_data!C9 &lt;Hib!A3,Hib!A3,Scenario_data!C9))</f>
-        <v>317824203.00978869</v>
+        <v>299210494.62320864</v>
       </c>
       <c r="D22" s="7">
         <f ca="1">IF(D9&gt;Hib!B4,Hib!B4,IF(Scenario_data!D9 &lt;Hib!A4,Hib!A4,Scenario_data!D9))</f>
-        <v>339636905.00294036</v>
+        <v>337698872.83373952</v>
       </c>
       <c r="E22" s="7">
         <f ca="1">IF(E9&gt;Hib!B5,Hib!B5,IF(Scenario_data!E9 &lt;Hib!A5,Hib!A5,Scenario_data!E9))</f>
-        <v>337903547.41550303</v>
+        <v>331646672.76028872</v>
       </c>
       <c r="F22" s="7">
         <f ca="1">IF(F9&gt;Hib!B6,Hib!B6,IF(Scenario_data!F9 &lt;Hib!A6,Hib!A6,Scenario_data!F9))</f>
-        <v>360246905.66393006</v>
+        <v>347464943.41047776</v>
       </c>
       <c r="G22" s="7">
         <f ca="1">IF(G9&gt;Hib!B7,Hib!B7,IF(Scenario_data!G9 &lt;Hib!A7,Hib!A7,Scenario_data!G9))</f>
-        <v>366909200.58424103</v>
+        <v>386705921.48365819</v>
       </c>
       <c r="H22" s="7">
         <f ca="1">IF(H9&gt;Hib!B8,Hib!B8,IF(Scenario_data!H9 &lt;Hib!A8,Hib!A8,Scenario_data!H9))</f>
-        <v>352892475.03423172</v>
+        <v>382836050.02938908</v>
       </c>
       <c r="I22" s="7">
         <f ca="1">IF(I9&gt;Hib!B9,Hib!B9,IF(Scenario_data!I9 &lt;Hib!A9,Hib!A9,Scenario_data!I9))</f>
-        <v>398952421.15679967</v>
+        <v>387186374.86042023</v>
       </c>
       <c r="J22" s="7">
         <f ca="1">IF(J9&gt;Hib!B10,Hib!B10,IF(Scenario_data!J9 &lt;Hib!A10,Hib!A10,Scenario_data!J9))</f>
-        <v>403596167.58389676</v>
+        <v>394100921.73965818</v>
       </c>
       <c r="K22" s="7">
         <f ca="1">IF(K9&gt;Hib!B11,Hib!B11,IF(Scenario_data!K9 &lt;Hib!A11,Hib!A11,Scenario_data!K9))</f>
-        <v>387444452.78617281</v>
+        <v>387291454.13088143</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
@@ -4048,43 +4063,43 @@
       </c>
       <c r="B23" s="7">
         <f ca="1">IF(B10&gt;Polio!B2,Polio!B2,IF(Scenario_data!B10 &lt;Polio!A2,Polio!A2,Scenario_data!B10))</f>
-        <v>716469135.2208643</v>
+        <v>652824044.21196711</v>
       </c>
       <c r="C23" s="7">
         <f ca="1">IF(C10&gt;Polio!B3,Polio!B3,IF(Scenario_data!C10 &lt;Polio!A3,Polio!A3,Scenario_data!C10))</f>
-        <v>609821971.85227132</v>
+        <v>690546743.04875004</v>
       </c>
       <c r="D23" s="7">
         <f ca="1">IF(D10&gt;Polio!B4,Polio!B4,IF(Scenario_data!D10 &lt;Polio!A4,Polio!A4,Scenario_data!D10))</f>
-        <v>695301475.81519341</v>
+        <v>692676867.17088211</v>
       </c>
       <c r="E23" s="7">
         <f ca="1">IF(E10&gt;Polio!B5,Polio!B5,IF(Scenario_data!E10 &lt;Polio!A5,Polio!A5,Scenario_data!E10))</f>
-        <v>762464447.93890333</v>
+        <v>654861721.33793247</v>
       </c>
       <c r="F23" s="7">
         <f ca="1">IF(F10&gt;Polio!B6,Polio!B6,IF(Scenario_data!F10 &lt;Polio!A6,Polio!A6,Scenario_data!F10))</f>
-        <v>686389314.4452064</v>
+        <v>700060601.90627897</v>
       </c>
       <c r="G23" s="7">
         <f ca="1">IF(G10&gt;Polio!B7,Polio!B7,IF(Scenario_data!G10 &lt;Polio!A7,Polio!A7,Scenario_data!G10))</f>
-        <v>799985931.68116021</v>
+        <v>798863703.98095632</v>
       </c>
       <c r="H23" s="7">
         <f ca="1">IF(H10&gt;Polio!B8,Polio!B8,IF(Scenario_data!H10 &lt;Polio!A8,Polio!A8,Scenario_data!H10))</f>
-        <v>831863821.14259303</v>
+        <v>879720173.04280317</v>
       </c>
       <c r="I23" s="7">
         <f ca="1">IF(I10&gt;Polio!B9,Polio!B9,IF(Scenario_data!I10 &lt;Polio!A9,Polio!A9,Scenario_data!I10))</f>
-        <v>873350186.74147618</v>
+        <v>887473998.43785214</v>
       </c>
       <c r="J23" s="7">
         <f ca="1">IF(J10&gt;Polio!B10,Polio!B10,IF(Scenario_data!J10 &lt;Polio!A10,Polio!A10,Scenario_data!J10))</f>
-        <v>816658245.66131377</v>
+        <v>836072319.12820292</v>
       </c>
       <c r="K23" s="7">
         <f ca="1">IF(K10&gt;Polio!B11,Polio!B11,IF(Scenario_data!K10 &lt;Polio!A11,Polio!A11,Scenario_data!K10))</f>
-        <v>962728529.51436865</v>
+        <v>986116583.99462807</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
@@ -4093,43 +4108,43 @@
       </c>
       <c r="B24" s="7">
         <f ca="1">IF(B11&gt;HPV!B2,HPV!B2,IF(Scenario_data!B11 &lt;HPV!A2,HPV!A2,Scenario_data!B11))</f>
-        <v>31963266.345840931</v>
+        <v>30560524.29243347</v>
       </c>
       <c r="C24" s="7">
         <f ca="1">IF(C11&gt;HPV!B3,HPV!B3,IF(Scenario_data!C11 &lt;HPV!A3,HPV!A3,Scenario_data!C11))</f>
-        <v>37221300.311860926</v>
+        <v>34918342.758120202</v>
       </c>
       <c r="D24" s="7">
         <f ca="1">IF(D11&gt;HPV!B4,HPV!B4,IF(Scenario_data!D11 &lt;HPV!A4,HPV!A4,Scenario_data!D11))</f>
-        <v>40900242.142210245</v>
+        <v>41436076.686650589</v>
       </c>
       <c r="E24" s="7">
         <f ca="1">IF(E11&gt;HPV!B5,HPV!B5,IF(Scenario_data!E11 &lt;HPV!A5,HPV!A5,Scenario_data!E11))</f>
-        <v>46648830.091460817</v>
+        <v>46040942.282288276</v>
       </c>
       <c r="F24" s="7">
         <f ca="1">IF(F11&gt;HPV!B6,HPV!B6,IF(Scenario_data!F11 &lt;HPV!A6,HPV!A6,Scenario_data!F11))</f>
-        <v>51958960.220131822</v>
+        <v>54828050.269251928</v>
       </c>
       <c r="G24" s="7">
         <f ca="1">IF(G11&gt;HPV!B7,HPV!B7,IF(Scenario_data!G11 &lt;HPV!A7,HPV!A7,Scenario_data!G11))</f>
-        <v>55169936.314006709</v>
+        <v>57301506.134691209</v>
       </c>
       <c r="H24" s="7">
         <f ca="1">IF(H11&gt;HPV!B8,HPV!B8,IF(Scenario_data!H11 &lt;HPV!A8,HPV!A8,Scenario_data!H11))</f>
-        <v>67707718.14164719</v>
+        <v>68291594.421742514</v>
       </c>
       <c r="I24" s="7">
         <f ca="1">IF(I11&gt;HPV!B9,HPV!B9,IF(Scenario_data!I11 &lt;HPV!A9,HPV!A9,Scenario_data!I11))</f>
-        <v>72924338.547077373</v>
+        <v>74993654.123364374</v>
       </c>
       <c r="J24" s="7">
         <f ca="1">IF(J11&gt;HPV!B10,HPV!B10,IF(Scenario_data!J11 &lt;HPV!A10,HPV!A10,Scenario_data!J11))</f>
-        <v>82191336.158397973</v>
+        <v>82144437.209521398</v>
       </c>
       <c r="K24" s="7">
         <f ca="1">IF(K11&gt;HPV!B11,HPV!B11,IF(Scenario_data!K11 &lt;HPV!A11,HPV!A11,Scenario_data!K11))</f>
-        <v>90347937.70977132</v>
+        <v>90825685.230482191</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
@@ -4138,43 +4153,43 @@
       </c>
       <c r="B25" s="7">
         <f ca="1">IF(B12&gt;Rotavirus!B2,Rotavirus!B2,IF(Scenario_data!B12 &lt;Rotavirus!A2,Rotavirus!A2,Scenario_data!B12))</f>
-        <v>180626332.14641702</v>
+        <v>187657992.33179039</v>
       </c>
       <c r="C25" s="7">
         <f ca="1">IF(C12&gt;Rotavirus!B3,Rotavirus!B3,IF(Scenario_data!C12 &lt;Rotavirus!A3,Rotavirus!A3,Scenario_data!C12))</f>
-        <v>234903455.59618309</v>
+        <v>225709798.05529684</v>
       </c>
       <c r="D25" s="7">
         <f ca="1">IF(D12&gt;Rotavirus!B4,Rotavirus!B4,IF(Scenario_data!D12 &lt;Rotavirus!A4,Rotavirus!A4,Scenario_data!D12))</f>
-        <v>251984068.42984644</v>
+        <v>210347798.03823003</v>
       </c>
       <c r="E25" s="7">
         <f ca="1">IF(E12&gt;Rotavirus!B5,Rotavirus!B5,IF(Scenario_data!E12 &lt;Rotavirus!A5,Rotavirus!A5,Scenario_data!E12))</f>
-        <v>239942103.58603629</v>
+        <v>280408646.42582417</v>
       </c>
       <c r="F25" s="7">
         <f ca="1">IF(F12&gt;Rotavirus!B6,Rotavirus!B6,IF(Scenario_data!F12 &lt;Rotavirus!A6,Rotavirus!A6,Scenario_data!F12))</f>
-        <v>344365641.33358532</v>
+        <v>309654253.49114066</v>
       </c>
       <c r="G25" s="7">
         <f ca="1">IF(G12&gt;Rotavirus!B7,Rotavirus!B7,IF(Scenario_data!G12 &lt;Rotavirus!A7,Rotavirus!A7,Scenario_data!G12))</f>
-        <v>377272561.38604409</v>
+        <v>358892927.70832986</v>
       </c>
       <c r="H25" s="7">
         <f ca="1">IF(H12&gt;Rotavirus!B8,Rotavirus!B8,IF(Scenario_data!H12 &lt;Rotavirus!A8,Rotavirus!A8,Scenario_data!H12))</f>
-        <v>423357966.73157269</v>
+        <v>439328951.17153937</v>
       </c>
       <c r="I25" s="7">
         <f ca="1">IF(I12&gt;Rotavirus!B9,Rotavirus!B9,IF(Scenario_data!I12 &lt;Rotavirus!A9,Rotavirus!A9,Scenario_data!I12))</f>
-        <v>567729050.62302148</v>
+        <v>540994027.48965824</v>
       </c>
       <c r="J25" s="7">
         <f ca="1">IF(J12&gt;Rotavirus!B10,Rotavirus!B10,IF(Scenario_data!J12 &lt;Rotavirus!A10,Rotavirus!A10,Scenario_data!J12))</f>
-        <v>605786630.78349292</v>
+        <v>622275062.8185575</v>
       </c>
       <c r="K25" s="7">
         <f ca="1">IF(K12&gt;Rotavirus!B11,Rotavirus!B11,IF(Scenario_data!K12 &lt;Rotavirus!A11,Rotavirus!A11,Scenario_data!K12))</f>
-        <v>791598901.25984669</v>
+        <v>740001258.35933352</v>
       </c>
       <c r="M25" s="4"/>
     </row>
@@ -4184,43 +4199,43 @@
       </c>
       <c r="B26" s="7">
         <f ca="1">IF(B13&gt;PCV!B2,PCV!B2,IF(Scenario_data!B13 &lt;PCV!A2,PCV!A2,Scenario_data!B13))</f>
-        <v>229617047.20396319</v>
+        <v>216802553.46174526</v>
       </c>
       <c r="C26" s="7">
         <f ca="1">IF(C13&gt;PCV!B3,PCV!B3,IF(Scenario_data!C13 &lt;PCV!A3,PCV!A3,Scenario_data!C13))</f>
-        <v>240945752.67308432</v>
+        <v>249520049.08285519</v>
       </c>
       <c r="D26" s="7">
         <f ca="1">IF(D13&gt;PCV!B4,PCV!B4,IF(Scenario_data!D13 &lt;PCV!A4,PCV!A4,Scenario_data!D13))</f>
-        <v>276233823.85737103</v>
+        <v>281047500.530514</v>
       </c>
       <c r="E26" s="7">
         <f ca="1">IF(E13&gt;PCV!B5,PCV!B5,IF(Scenario_data!E13 &lt;PCV!A5,PCV!A5,Scenario_data!E13))</f>
-        <v>314594025.93042862</v>
+        <v>319452704.40594953</v>
       </c>
       <c r="F26" s="7">
         <f ca="1">IF(F13&gt;PCV!B6,PCV!B6,IF(Scenario_data!F13 &lt;PCV!A6,PCV!A6,Scenario_data!F13))</f>
-        <v>321897015.9009065</v>
+        <v>340266975.06073743</v>
       </c>
       <c r="G26" s="7">
         <f ca="1">IF(G13&gt;PCV!B7,PCV!B7,IF(Scenario_data!G13 &lt;PCV!A7,PCV!A7,Scenario_data!G13))</f>
-        <v>386260327.82587272</v>
+        <v>369787155.59154975</v>
       </c>
       <c r="H26" s="7">
         <f ca="1">IF(H13&gt;PCV!B8,PCV!B8,IF(Scenario_data!H13 &lt;PCV!A8,PCV!A8,Scenario_data!H13))</f>
-        <v>405501499.43285483</v>
+        <v>410950595.54557264</v>
       </c>
       <c r="I26" s="7">
         <f ca="1">IF(I13&gt;PCV!B9,PCV!B9,IF(Scenario_data!I13 &lt;PCV!A9,PCV!A9,Scenario_data!I13))</f>
-        <v>458134082.10548717</v>
+        <v>451215498.21884525</v>
       </c>
       <c r="J26" s="7">
         <f ca="1">IF(J13&gt;PCV!B10,PCV!B10,IF(Scenario_data!J13 &lt;PCV!A10,PCV!A10,Scenario_data!J13))</f>
-        <v>470477084.71559083</v>
+        <v>504019857.09622318</v>
       </c>
       <c r="K26" s="7">
         <f ca="1">IF(K13&gt;PCV!B11,PCV!B11,IF(Scenario_data!K13 &lt;PCV!A11,PCV!A11,Scenario_data!K13))</f>
-        <v>428131633.6187433</v>
+        <v>424042535.01040512</v>
       </c>
       <c r="M26" s="4"/>
     </row>

</xml_diff>